<commit_message>
SeccionOficio: reducir padding inferior en móvil (pb-8) para acercar el botón a la wincha, igual que en desktop; desktop sin cambios
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_precios/Consolidado_lista_de_precios_2026_.xlsx
+++ b/_precios/Consolidado_lista_de_precios_2026_.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elcapel/Library/CloudStorage/GoogleDrive-garcia.persi@gmail.com/Mi unidad/KPL_BRANDING/Clientes/Devas/velas-devas/_precios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C85ED6-8B7F-F34C-B891-F81DE62AC98E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AECE92A-1A95-F149-8207-A935E826E258}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30220" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="600" windowWidth="38400" windowHeight="21000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONSOLIDADO" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="283">
   <si>
     <t>PANTALLAS</t>
   </si>
@@ -649,13 +649,7 @@
     <t>VD059</t>
   </si>
   <si>
-    <t>Vela Bautizo</t>
-  </si>
-  <si>
     <t>VD060</t>
-  </si>
-  <si>
-    <t>Vela Bautizo color</t>
   </si>
   <si>
     <t>VD061</t>
@@ -902,7 +896,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -942,6 +936,13 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1234,7 +1235,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1306,6 +1307,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1621,7 +1625,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E201"/>
+  <dimension ref="A1:E198"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.5" customWidth="1"/>
@@ -1678,7 +1682,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>83</v>
@@ -1696,8 +1700,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>281</v>
+      <c r="A6" s="30" t="s">
+        <v>279</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>84</v>
@@ -1772,7 +1776,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="30" t="s">
         <v>91</v>
       </c>
       <c r="B10" s="4" t="s">
@@ -1791,7 +1795,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="30" t="s">
         <v>93</v>
       </c>
       <c r="B11" s="4" t="s">
@@ -1810,7 +1814,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="30" t="s">
         <v>95</v>
       </c>
       <c r="B12" s="4" t="s">
@@ -1829,7 +1833,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="30" t="s">
         <v>97</v>
       </c>
       <c r="B13" s="4" t="s">
@@ -2285,7 +2289,7 @@
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" s="3" t="s">
+      <c r="A44" s="30" t="s">
         <v>145</v>
       </c>
       <c r="B44" s="4" t="s">
@@ -2304,7 +2308,7 @@
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" s="3" t="s">
+      <c r="A45" s="30" t="s">
         <v>147</v>
       </c>
       <c r="B45" s="4" t="s">
@@ -2835,126 +2839,128 @@
         <v>20944</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A78" s="8" t="s">
+    <row r="77" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A78" s="26" t="s">
+        <v>205</v>
+      </c>
+      <c r="B78" s="27"/>
+      <c r="C78" s="27"/>
+      <c r="D78" s="27"/>
+      <c r="E78" s="28"/>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A79" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D79" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E79" s="7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A80" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="C80" s="5">
+        <v>2200</v>
+      </c>
+      <c r="D80" s="5">
+        <f>C80*19%</f>
+        <v>418</v>
+      </c>
+      <c r="E80" s="9">
+        <f>C80+D80</f>
+        <v>2618</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A81" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C81" s="5">
+        <v>2400</v>
+      </c>
+      <c r="D81" s="5">
+        <f>C81*19%</f>
+        <v>456</v>
+      </c>
+      <c r="E81" s="9">
+        <f>C81+D81</f>
+        <v>2856</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A82" s="8" t="s">
         <v>282</v>
       </c>
-      <c r="B78" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="C78" s="5">
-        <v>2200</v>
-      </c>
-      <c r="D78" s="5">
-        <f>C78*19%</f>
-        <v>418</v>
-      </c>
-      <c r="E78" s="5">
-        <f>C78+D78</f>
-        <v>2618</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A79" s="8" t="s">
-        <v>283</v>
-      </c>
-      <c r="B79" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="C79" s="5">
-        <v>2400</v>
-      </c>
-      <c r="D79" s="5">
-        <f>C79*19%</f>
-        <v>456</v>
-      </c>
-      <c r="E79" s="5">
-        <f>C79+D79</f>
-        <v>2856</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="26" t="s">
+      <c r="B82" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="B81" s="27"/>
-      <c r="C81" s="27"/>
-      <c r="D81" s="27"/>
-      <c r="E81" s="28"/>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A82" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E82" s="7" t="s">
-        <v>5</v>
+      <c r="C82" s="5">
+        <v>1850</v>
+      </c>
+      <c r="D82" s="5">
+        <f>C82*19%</f>
+        <v>351.5</v>
+      </c>
+      <c r="E82" s="9">
+        <f>C82+D82</f>
+        <v>2201.5</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" s="8" t="s">
-        <v>282</v>
+        <v>208</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="C83" s="5">
-        <v>2200</v>
+        <v>4600</v>
       </c>
       <c r="D83" s="5">
         <f>C83*19%</f>
-        <v>418</v>
+        <v>874</v>
       </c>
       <c r="E83" s="9">
         <f>C83+D83</f>
-        <v>2618</v>
+        <v>5474</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A84" s="8" t="s">
-        <v>283</v>
-      </c>
-      <c r="B84" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="C84" s="5">
-        <v>2400</v>
-      </c>
-      <c r="D84" s="5">
-        <f>C84*19%</f>
-        <v>456</v>
-      </c>
-      <c r="E84" s="9">
-        <f>C84+D84</f>
-        <v>2856</v>
-      </c>
+      <c r="A84" s="1"/>
+      <c r="E84" s="10"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A85" s="8" t="s">
-        <v>284</v>
-      </c>
-      <c r="B85" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="C85" s="5">
-        <v>1850</v>
-      </c>
-      <c r="D85" s="5">
-        <f>C85*19%</f>
-        <v>351.5</v>
-      </c>
-      <c r="E85" s="9">
-        <f>C85+D85</f>
-        <v>2201.5</v>
+      <c r="A85" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E85" s="7" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.2">
@@ -2965,308 +2971,308 @@
         <v>211</v>
       </c>
       <c r="C86" s="5">
-        <v>4600</v>
+        <v>2350</v>
       </c>
       <c r="D86" s="5">
         <f>C86*19%</f>
-        <v>874</v>
+        <v>446.5</v>
       </c>
       <c r="E86" s="9">
         <f>C86+D86</f>
-        <v>5474</v>
+        <v>2796.5</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A87" s="1"/>
-      <c r="E87" s="10"/>
+      <c r="A87" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="C87" s="5">
+        <v>2830</v>
+      </c>
+      <c r="D87" s="5">
+        <f>C87*19%</f>
+        <v>537.70000000000005</v>
+      </c>
+      <c r="E87" s="9">
+        <f>C87+D87</f>
+        <v>3367.7</v>
+      </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A88" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C88" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D88" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E88" s="7" t="s">
-        <v>5</v>
+      <c r="A88" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="C88" s="5">
+        <v>3300</v>
+      </c>
+      <c r="D88" s="5">
+        <f>C88*19%</f>
+        <v>627</v>
+      </c>
+      <c r="E88" s="9">
+        <f>C88+D88</f>
+        <v>3927</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89" s="8" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C89" s="5">
-        <v>2350</v>
+        <v>3850</v>
       </c>
       <c r="D89" s="5">
         <f>C89*19%</f>
-        <v>446.5</v>
+        <v>731.5</v>
       </c>
       <c r="E89" s="9">
         <f>C89+D89</f>
-        <v>2796.5</v>
+        <v>4581.5</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A90" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="B90" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="C90" s="5">
-        <v>2830</v>
-      </c>
-      <c r="D90" s="5">
-        <f>C90*19%</f>
-        <v>537.70000000000005</v>
-      </c>
-      <c r="E90" s="9">
-        <f>C90+D90</f>
-        <v>3367.7</v>
-      </c>
+      <c r="A90" s="1"/>
+      <c r="E90" s="10"/>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A91" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="B91" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="C91" s="5">
-        <v>3300</v>
-      </c>
-      <c r="D91" s="5">
-        <f>C91*19%</f>
-        <v>627</v>
-      </c>
-      <c r="E91" s="9">
-        <f>C91+D91</f>
-        <v>3927</v>
-      </c>
+      <c r="A91" s="1"/>
+      <c r="E91" s="10"/>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A92" s="8" t="s">
+      <c r="A92" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E92" s="7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A93" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="B92" s="4" t="s">
+      <c r="B93" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="C92" s="5">
-        <v>3850</v>
-      </c>
-      <c r="D92" s="5">
-        <f>C92*19%</f>
-        <v>731.5</v>
-      </c>
-      <c r="E92" s="9">
-        <f>C92+D92</f>
-        <v>4581.5</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A93" s="1"/>
-      <c r="E93" s="10"/>
+      <c r="C93" s="5">
+        <v>7810</v>
+      </c>
+      <c r="D93" s="5">
+        <f t="shared" ref="D93:D102" si="10">C93*19%</f>
+        <v>1483.9</v>
+      </c>
+      <c r="E93" s="9">
+        <f t="shared" ref="E93:E102" si="11">C93+D93</f>
+        <v>9293.9</v>
+      </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A94" s="1"/>
-      <c r="E94" s="10"/>
+      <c r="A94" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="C94" s="5">
+        <v>8900</v>
+      </c>
+      <c r="D94" s="5">
+        <f t="shared" si="10"/>
+        <v>1691</v>
+      </c>
+      <c r="E94" s="9">
+        <f t="shared" si="11"/>
+        <v>10591</v>
+      </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A95" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B95" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C95" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D95" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E95" s="7" t="s">
-        <v>5</v>
+      <c r="A95" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="C95" s="5">
+        <v>10400</v>
+      </c>
+      <c r="D95" s="5">
+        <f t="shared" si="10"/>
+        <v>1976</v>
+      </c>
+      <c r="E95" s="9">
+        <f t="shared" si="11"/>
+        <v>12376</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96" s="8" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C96" s="5">
-        <v>7810</v>
+        <v>12000</v>
       </c>
       <c r="D96" s="5">
-        <f t="shared" ref="D96:D105" si="10">C96*19%</f>
-        <v>1483.9</v>
+        <f t="shared" si="10"/>
+        <v>2280</v>
       </c>
       <c r="E96" s="9">
-        <f t="shared" ref="E96:E105" si="11">C96+D96</f>
-        <v>9293.9</v>
+        <f t="shared" si="11"/>
+        <v>14280</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97" s="8" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="C97" s="5">
-        <v>8900</v>
+        <v>19300</v>
       </c>
       <c r="D97" s="5">
         <f t="shared" si="10"/>
-        <v>1691</v>
+        <v>3667</v>
       </c>
       <c r="E97" s="9">
         <f t="shared" si="11"/>
-        <v>10591</v>
+        <v>22967</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98" s="8" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C98" s="5">
-        <v>10400</v>
+        <v>22500</v>
       </c>
       <c r="D98" s="5">
         <f t="shared" si="10"/>
-        <v>1976</v>
+        <v>4275</v>
       </c>
       <c r="E98" s="9">
         <f t="shared" si="11"/>
-        <v>12376</v>
+        <v>26775</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99" s="8" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C99" s="5">
-        <v>12000</v>
+        <v>26400</v>
       </c>
       <c r="D99" s="5">
         <f t="shared" si="10"/>
-        <v>2280</v>
+        <v>5016</v>
       </c>
       <c r="E99" s="9">
         <f t="shared" si="11"/>
-        <v>14280</v>
+        <v>31416</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100" s="8" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C100" s="5">
-        <v>19300</v>
+        <v>28500</v>
       </c>
       <c r="D100" s="5">
         <f t="shared" si="10"/>
-        <v>3667</v>
+        <v>5415</v>
       </c>
       <c r="E100" s="9">
         <f t="shared" si="11"/>
-        <v>22967</v>
+        <v>33915</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101" s="8" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="C101" s="5">
-        <v>22500</v>
+        <v>31680</v>
       </c>
       <c r="D101" s="5">
         <f t="shared" si="10"/>
-        <v>4275</v>
+        <v>6019.2</v>
       </c>
       <c r="E101" s="9">
         <f t="shared" si="11"/>
-        <v>26775</v>
+        <v>37699.199999999997</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102" s="8" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C102" s="5">
-        <v>26400</v>
+        <v>40150</v>
       </c>
       <c r="D102" s="5">
         <f t="shared" si="10"/>
-        <v>5016</v>
+        <v>7628.5</v>
       </c>
       <c r="E102" s="9">
         <f t="shared" si="11"/>
-        <v>31416</v>
+        <v>47778.5</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A103" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="B103" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="C103" s="5">
-        <v>28500</v>
-      </c>
-      <c r="D103" s="5">
-        <f t="shared" si="10"/>
-        <v>5415</v>
-      </c>
-      <c r="E103" s="9">
-        <f t="shared" si="11"/>
-        <v>33915</v>
-      </c>
+      <c r="A103" s="1"/>
+      <c r="E103" s="10"/>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A104" s="8" t="s">
-        <v>236</v>
-      </c>
-      <c r="B104" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="C104" s="5">
-        <v>31680</v>
-      </c>
-      <c r="D104" s="5">
-        <f t="shared" si="10"/>
-        <v>6019.2</v>
-      </c>
-      <c r="E104" s="9">
-        <f t="shared" si="11"/>
-        <v>37699.199999999997</v>
+      <c r="A104" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E104" s="7" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
@@ -3277,131 +3283,131 @@
         <v>239</v>
       </c>
       <c r="C105" s="5">
-        <v>40150</v>
+        <v>17500</v>
       </c>
       <c r="D105" s="5">
-        <f t="shared" si="10"/>
-        <v>7628.5</v>
+        <f t="shared" ref="D105:D110" si="12">C105*19%</f>
+        <v>3325</v>
       </c>
       <c r="E105" s="9">
-        <f t="shared" si="11"/>
-        <v>47778.5</v>
+        <f t="shared" ref="E105:E110" si="13">C105+D105</f>
+        <v>20825</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A106" s="1"/>
-      <c r="E106" s="10"/>
+      <c r="A106" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="C106" s="5">
+        <v>25800</v>
+      </c>
+      <c r="D106" s="5">
+        <f t="shared" si="12"/>
+        <v>4902</v>
+      </c>
+      <c r="E106" s="9">
+        <f t="shared" si="13"/>
+        <v>30702</v>
+      </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A107" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C107" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D107" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E107" s="7" t="s">
-        <v>5</v>
+      <c r="A107" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="C107" s="5">
+        <v>29850</v>
+      </c>
+      <c r="D107" s="5">
+        <f t="shared" si="12"/>
+        <v>5671.5</v>
+      </c>
+      <c r="E107" s="9">
+        <f t="shared" si="13"/>
+        <v>35521.5</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108" s="8" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C108" s="5">
-        <v>17500</v>
+        <v>32890</v>
       </c>
       <c r="D108" s="5">
-        <f t="shared" ref="D108:D113" si="12">C108*19%</f>
-        <v>3325</v>
+        <f t="shared" si="12"/>
+        <v>6249.1</v>
       </c>
       <c r="E108" s="9">
-        <f t="shared" ref="E108:E113" si="13">C108+D108</f>
-        <v>20825</v>
+        <f t="shared" si="13"/>
+        <v>39139.1</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109" s="8" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C109" s="5">
-        <v>25800</v>
+        <v>38610</v>
       </c>
       <c r="D109" s="5">
         <f t="shared" si="12"/>
-        <v>4902</v>
+        <v>7335.9</v>
       </c>
       <c r="E109" s="9">
         <f t="shared" si="13"/>
-        <v>30702</v>
+        <v>45945.9</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110" s="8" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="C110" s="5">
-        <v>29850</v>
+        <v>48620</v>
       </c>
       <c r="D110" s="5">
         <f t="shared" si="12"/>
-        <v>5671.5</v>
+        <v>9237.7999999999993</v>
       </c>
       <c r="E110" s="9">
         <f t="shared" si="13"/>
-        <v>35521.5</v>
+        <v>57857.8</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A111" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="B111" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="C111" s="5">
-        <v>32890</v>
-      </c>
-      <c r="D111" s="5">
-        <f t="shared" si="12"/>
-        <v>6249.1</v>
-      </c>
-      <c r="E111" s="9">
-        <f t="shared" si="13"/>
-        <v>39139.1</v>
-      </c>
+      <c r="A111" s="1"/>
+      <c r="E111" s="10"/>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A112" s="8" t="s">
-        <v>248</v>
-      </c>
-      <c r="B112" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="C112" s="5">
-        <v>38610</v>
-      </c>
-      <c r="D112" s="5">
-        <f t="shared" si="12"/>
-        <v>7335.9</v>
-      </c>
-      <c r="E112" s="9">
-        <f t="shared" si="13"/>
-        <v>45945.9</v>
+      <c r="A112" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E112" s="7" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.2">
@@ -3412,1412 +3418,1372 @@
         <v>251</v>
       </c>
       <c r="C113" s="5">
-        <v>48620</v>
+        <v>55600</v>
       </c>
       <c r="D113" s="5">
-        <f t="shared" si="12"/>
-        <v>9237.7999999999993</v>
+        <f>C113*19%</f>
+        <v>10564</v>
       </c>
       <c r="E113" s="9">
-        <f t="shared" si="13"/>
-        <v>57857.8</v>
+        <f>C113+D113</f>
+        <v>66164</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A114" s="1"/>
-      <c r="E114" s="10"/>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A115" s="6" t="s">
+      <c r="A114" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="C114" s="5">
+        <v>60100</v>
+      </c>
+      <c r="D114" s="5">
+        <f>C114*19%</f>
+        <v>11419</v>
+      </c>
+      <c r="E114" s="9">
+        <f>C114+D114</f>
+        <v>71519</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A116" s="23" t="s">
+        <v>254</v>
+      </c>
+      <c r="B116" s="24"/>
+      <c r="C116" s="24"/>
+      <c r="D116" s="24"/>
+      <c r="E116" s="25"/>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A117" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B115" s="2" t="s">
+      <c r="B117" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C115" s="2" t="s">
+      <c r="C117" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D115" s="2" t="s">
+      <c r="D117" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E115" s="7" t="s">
+      <c r="E117" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A116" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="B116" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="C116" s="5">
-        <v>55600</v>
-      </c>
-      <c r="D116" s="5">
-        <f>C116*19%</f>
-        <v>10564</v>
-      </c>
-      <c r="E116" s="9">
-        <f>C116+D116</f>
-        <v>66164</v>
-      </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A117" s="8" t="s">
-        <v>254</v>
-      </c>
-      <c r="B117" s="4" t="s">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A118" s="8" t="s">
+        <v>206</v>
+      </c>
+      <c r="B118" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="C117" s="5">
-        <v>60100</v>
-      </c>
-      <c r="D117" s="5">
-        <f>C117*19%</f>
-        <v>11419</v>
-      </c>
-      <c r="E117" s="9">
-        <f>C117+D117</f>
-        <v>71519</v>
-      </c>
-    </row>
-    <row r="119" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A119" s="23" t="s">
+      <c r="C118" s="5">
+        <v>1500</v>
+      </c>
+      <c r="D118" s="5">
+        <f>C118*19%</f>
+        <v>285</v>
+      </c>
+      <c r="E118" s="9">
+        <f>C118+D118</f>
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A119" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="B119" s="24"/>
-      <c r="C119" s="24"/>
-      <c r="D119" s="24"/>
-      <c r="E119" s="25"/>
+      <c r="B119" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="C119" s="5">
+        <v>2600</v>
+      </c>
+      <c r="D119" s="5">
+        <f>C119*19%</f>
+        <v>494</v>
+      </c>
+      <c r="E119" s="9">
+        <f>C119+D119</f>
+        <v>3094</v>
+      </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A120" s="6" t="s">
+      <c r="A120" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="C120" s="5">
+        <v>3700</v>
+      </c>
+      <c r="D120" s="5">
+        <f>C120*19%</f>
+        <v>703</v>
+      </c>
+      <c r="E120" s="9">
+        <f>C120+D120</f>
+        <v>4403</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A121" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="B121" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="C121" s="13">
+        <v>6500</v>
+      </c>
+      <c r="D121" s="13">
+        <f>C121*19%</f>
+        <v>1235</v>
+      </c>
+      <c r="E121" s="14">
+        <f>C121+D121</f>
+        <v>7735</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="123" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A123" s="20" t="s">
+        <v>260</v>
+      </c>
+      <c r="B123" s="21"/>
+      <c r="C123" s="21"/>
+      <c r="D123" s="21"/>
+      <c r="E123" s="22"/>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A124" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B120" s="2" t="s">
+      <c r="B124" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C120" s="2" t="s">
+      <c r="C124" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="D120" s="2" t="s">
+      <c r="D124" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E120" s="7" t="s">
+      <c r="E124" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A121" s="8" t="s">
-        <v>208</v>
-      </c>
-      <c r="B121" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="C121" s="5">
-        <v>1500</v>
-      </c>
-      <c r="D121" s="5">
-        <f>C121*19%</f>
-        <v>285</v>
-      </c>
-      <c r="E121" s="9">
-        <f>C121+D121</f>
-        <v>1785</v>
-      </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A122" s="8" t="s">
-        <v>258</v>
-      </c>
-      <c r="B122" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="C122" s="5">
-        <v>2600</v>
-      </c>
-      <c r="D122" s="5">
-        <f>C122*19%</f>
-        <v>494</v>
-      </c>
-      <c r="E122" s="9">
-        <f>C122+D122</f>
-        <v>3094</v>
-      </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A123" s="8" t="s">
-        <v>210</v>
-      </c>
-      <c r="B123" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="C123" s="5">
-        <v>3700</v>
-      </c>
-      <c r="D123" s="5">
-        <f>C123*19%</f>
-        <v>703</v>
-      </c>
-      <c r="E123" s="9">
-        <f>C123+D123</f>
-        <v>4403</v>
-      </c>
-    </row>
-    <row r="124" spans="1:5" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="11" t="s">
-        <v>222</v>
-      </c>
-      <c r="B124" s="12" t="s">
-        <v>261</v>
-      </c>
-      <c r="C124" s="13">
-        <v>6500</v>
-      </c>
-      <c r="D124" s="13">
-        <f>C124*19%</f>
-        <v>1235</v>
-      </c>
-      <c r="E124" s="14">
-        <f>C124+D124</f>
-        <v>7735</v>
-      </c>
-    </row>
-    <row r="125" spans="1:5" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A126" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="B126" s="21"/>
-      <c r="C126" s="21"/>
-      <c r="D126" s="21"/>
-      <c r="E126" s="22"/>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A127" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="B127" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="C127" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="D127" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E127" s="2" t="s">
-        <v>5</v>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A125" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C125" s="5">
+        <v>330</v>
+      </c>
+      <c r="D125" s="5">
+        <f>C125*19%</f>
+        <v>62.7</v>
+      </c>
+      <c r="E125" s="5">
+        <f>C125+D125</f>
+        <v>392.7</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A126" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C126" s="5">
+        <v>410</v>
+      </c>
+      <c r="D126" s="5">
+        <f>C126*19%</f>
+        <v>77.900000000000006</v>
+      </c>
+      <c r="E126" s="5">
+        <f>C126+D126</f>
+        <v>487.9</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A128" s="3" t="s">
-        <v>280</v>
+        <v>85</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C128" s="5">
-        <v>330</v>
+        <v>580</v>
       </c>
       <c r="D128" s="5">
-        <f>C128*19%</f>
-        <v>62.7</v>
+        <f t="shared" ref="D128:D135" si="14">C128*19%</f>
+        <v>110.2</v>
       </c>
       <c r="E128" s="5">
-        <f>C128+D128</f>
-        <v>392.7</v>
+        <f t="shared" ref="E128:E135" si="15">C128+D128</f>
+        <v>690.2</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A129" s="3" t="s">
-        <v>281</v>
+        <v>87</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C129" s="5">
-        <v>410</v>
+        <v>890</v>
       </c>
       <c r="D129" s="5">
-        <f>C129*19%</f>
-        <v>77.900000000000006</v>
+        <f t="shared" si="14"/>
+        <v>169.1</v>
       </c>
       <c r="E129" s="5">
-        <f>C129+D129</f>
-        <v>487.9</v>
+        <f t="shared" si="15"/>
+        <v>1059.0999999999999</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A130" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C130" s="5">
+        <v>1350</v>
+      </c>
+      <c r="D130" s="5">
+        <f t="shared" si="14"/>
+        <v>256.5</v>
+      </c>
+      <c r="E130" s="5">
+        <f t="shared" si="15"/>
+        <v>1606.5</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131" s="3" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C131" s="5">
-        <v>580</v>
+        <v>1420</v>
       </c>
       <c r="D131" s="5">
-        <f t="shared" ref="D131:D138" si="14">C131*19%</f>
-        <v>110.2</v>
+        <f t="shared" si="14"/>
+        <v>269.8</v>
       </c>
       <c r="E131" s="5">
-        <f t="shared" ref="E131:E138" si="15">C131+D131</f>
-        <v>690.2</v>
+        <f t="shared" si="15"/>
+        <v>1689.8</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132" s="3" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C132" s="5">
-        <v>890</v>
+        <v>2000</v>
       </c>
       <c r="D132" s="5">
         <f t="shared" si="14"/>
-        <v>169.1</v>
+        <v>380</v>
       </c>
       <c r="E132" s="5">
         <f t="shared" si="15"/>
-        <v>1059.0999999999999</v>
+        <v>2380</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A133" s="3" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="C133" s="5">
-        <v>1350</v>
+        <v>2400</v>
       </c>
       <c r="D133" s="5">
         <f t="shared" si="14"/>
-        <v>256.5</v>
+        <v>456</v>
       </c>
       <c r="E133" s="5">
         <f t="shared" si="15"/>
-        <v>1606.5</v>
+        <v>2856</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A134" s="3" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C134" s="5">
-        <v>1420</v>
+        <v>2600</v>
       </c>
       <c r="D134" s="5">
         <f t="shared" si="14"/>
-        <v>269.8</v>
+        <v>494</v>
       </c>
       <c r="E134" s="5">
         <f t="shared" si="15"/>
-        <v>1689.8</v>
+        <v>3094</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A135" s="3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C135" s="5">
-        <v>2000</v>
+        <v>3580</v>
       </c>
       <c r="D135" s="5">
         <f t="shared" si="14"/>
-        <v>380</v>
+        <v>680.2</v>
       </c>
       <c r="E135" s="5">
         <f t="shared" si="15"/>
-        <v>2380</v>
-      </c>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A136" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B136" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C136" s="5">
-        <v>2400</v>
-      </c>
-      <c r="D136" s="5">
-        <f t="shared" si="14"/>
-        <v>456</v>
-      </c>
-      <c r="E136" s="5">
-        <f t="shared" si="15"/>
-        <v>2856</v>
+        <v>4260.2</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A137" s="3" t="s">
-        <v>97</v>
+        <v>141</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>98</v>
+        <v>142</v>
       </c>
       <c r="C137" s="5">
-        <v>2600</v>
+        <v>2200</v>
       </c>
       <c r="D137" s="5">
-        <f t="shared" si="14"/>
-        <v>494</v>
+        <f>C137*19%</f>
+        <v>418</v>
       </c>
       <c r="E137" s="5">
-        <f t="shared" si="15"/>
-        <v>3094</v>
+        <f>C137+D137</f>
+        <v>2618</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A138" s="3" t="s">
-        <v>99</v>
+        <v>143</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>100</v>
+        <v>144</v>
       </c>
       <c r="C138" s="5">
-        <v>3580</v>
+        <v>2750</v>
       </c>
       <c r="D138" s="5">
-        <f t="shared" si="14"/>
-        <v>680.2</v>
+        <f>C138*19%</f>
+        <v>522.5</v>
       </c>
       <c r="E138" s="5">
-        <f t="shared" si="15"/>
-        <v>4260.2</v>
-      </c>
-    </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A140" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="B140" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="C140" s="5">
-        <v>2200</v>
-      </c>
-      <c r="D140" s="5">
-        <f>C140*19%</f>
-        <v>418</v>
-      </c>
-      <c r="E140" s="5">
-        <f>C140+D140</f>
-        <v>2618</v>
+        <f>C138+D138</f>
+        <v>3272.5</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A139" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C139" s="5">
+        <v>4500</v>
+      </c>
+      <c r="D139" s="5">
+        <f>C139*19%</f>
+        <v>855</v>
+      </c>
+      <c r="E139" s="5">
+        <f>C139+D139</f>
+        <v>5355</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A141" s="3" t="s">
-        <v>143</v>
+        <v>165</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="C141" s="5">
-        <v>2750</v>
+        <v>1550</v>
       </c>
       <c r="D141" s="5">
         <f>C141*19%</f>
-        <v>522.5</v>
+        <v>294.5</v>
       </c>
       <c r="E141" s="5">
         <f>C141+D141</f>
-        <v>3272.5</v>
-      </c>
-    </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A142" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="B142" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="C142" s="5">
-        <v>4500</v>
-      </c>
-      <c r="D142" s="5">
-        <f>C142*19%</f>
-        <v>855</v>
-      </c>
-      <c r="E142" s="5">
-        <f>C142+D142</f>
-        <v>5355</v>
+        <v>1844.5</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A144" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="B144" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="C144" s="5">
-        <v>1550</v>
+      <c r="A144" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="B144" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C144" s="17">
+        <v>480</v>
       </c>
       <c r="D144" s="5">
         <f>C144*19%</f>
-        <v>294.5</v>
+        <v>91.2</v>
       </c>
       <c r="E144" s="5">
         <f>C144+D144</f>
-        <v>1844.5</v>
-      </c>
-    </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A147" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="B147" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="C147" s="17">
-        <v>480</v>
-      </c>
-      <c r="D147" s="5">
-        <f>C147*19%</f>
-        <v>91.2</v>
-      </c>
-      <c r="E147" s="5">
-        <f>C147+D147</f>
         <v>571.20000000000005</v>
       </c>
     </row>
-    <row r="152" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A152" s="23" t="s">
+    <row r="149" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A149" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B152" s="24"/>
-      <c r="C152" s="24"/>
-      <c r="D152" s="24"/>
-      <c r="E152" s="25"/>
+      <c r="B149" s="24"/>
+      <c r="C149" s="24"/>
+      <c r="D149" s="24"/>
+      <c r="E149" s="25"/>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A150" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B150" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="C150" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E150" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A151" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B151" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C151" s="5">
+        <v>1600</v>
+      </c>
+      <c r="D151" s="5">
+        <f t="shared" ref="D151:D187" si="16">C151*19%</f>
+        <v>304</v>
+      </c>
+      <c r="E151" s="9">
+        <f t="shared" ref="E151:E187" si="17">C151+D151</f>
+        <v>1904</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A152" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B152" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C152" s="5">
+        <v>2800</v>
+      </c>
+      <c r="D152" s="5">
+        <f t="shared" si="16"/>
+        <v>532</v>
+      </c>
+      <c r="E152" s="9">
+        <f t="shared" si="17"/>
+        <v>3332</v>
+      </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A153" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="B153" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="C153" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="D153" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E153" s="2" t="s">
-        <v>5</v>
+      <c r="A153" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B153" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C153" s="5">
+        <v>3400</v>
+      </c>
+      <c r="D153" s="5">
+        <f t="shared" si="16"/>
+        <v>646</v>
+      </c>
+      <c r="E153" s="9">
+        <f t="shared" si="17"/>
+        <v>4046</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A154" s="8" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C154" s="5">
-        <v>1600</v>
+        <v>4100</v>
       </c>
       <c r="D154" s="5">
-        <f t="shared" ref="D154:D190" si="16">C154*19%</f>
-        <v>304</v>
+        <f t="shared" si="16"/>
+        <v>779</v>
       </c>
       <c r="E154" s="9">
-        <f t="shared" ref="E154:E190" si="17">C154+D154</f>
-        <v>1904</v>
+        <f t="shared" si="17"/>
+        <v>4879</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A155" s="8" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C155" s="5">
-        <v>2800</v>
+        <v>5300</v>
       </c>
       <c r="D155" s="5">
         <f t="shared" si="16"/>
-        <v>532</v>
+        <v>1007</v>
       </c>
       <c r="E155" s="9">
         <f t="shared" si="17"/>
-        <v>3332</v>
+        <v>6307</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A156" s="8" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C156" s="5">
-        <v>3400</v>
+        <v>5800</v>
       </c>
       <c r="D156" s="5">
         <f t="shared" si="16"/>
-        <v>646</v>
+        <v>1102</v>
       </c>
       <c r="E156" s="9">
         <f t="shared" si="17"/>
-        <v>4046</v>
+        <v>6902</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A157" s="8" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C157" s="5">
-        <v>4100</v>
+        <v>5950</v>
       </c>
       <c r="D157" s="5">
         <f t="shared" si="16"/>
-        <v>779</v>
+        <v>1130.5</v>
       </c>
       <c r="E157" s="9">
         <f t="shared" si="17"/>
-        <v>4879</v>
+        <v>7080.5</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A158" s="8" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B158" s="4" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C158" s="5">
-        <v>5300</v>
+        <v>9100</v>
       </c>
       <c r="D158" s="5">
         <f t="shared" si="16"/>
-        <v>1007</v>
+        <v>1729</v>
       </c>
       <c r="E158" s="9">
         <f t="shared" si="17"/>
-        <v>6307</v>
+        <v>10829</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A159" s="8" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C159" s="5">
-        <v>5800</v>
+        <v>14850</v>
       </c>
       <c r="D159" s="5">
         <f t="shared" si="16"/>
-        <v>1102</v>
+        <v>2821.5</v>
       </c>
       <c r="E159" s="9">
         <f t="shared" si="17"/>
-        <v>6902</v>
+        <v>17671.5</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A160" s="8" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B160" s="4" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C160" s="5">
-        <v>5950</v>
+        <v>19800</v>
       </c>
       <c r="D160" s="5">
         <f t="shared" si="16"/>
-        <v>1130.5</v>
+        <v>3762</v>
       </c>
       <c r="E160" s="9">
         <f t="shared" si="17"/>
-        <v>7080.5</v>
+        <v>23562</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A161" s="8" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B161" s="4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C161" s="5">
-        <v>9100</v>
+        <v>15200</v>
       </c>
       <c r="D161" s="5">
         <f t="shared" si="16"/>
-        <v>1729</v>
+        <v>2888</v>
       </c>
       <c r="E161" s="9">
         <f t="shared" si="17"/>
-        <v>10829</v>
+        <v>18088</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A162" s="8" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B162" s="4" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C162" s="5">
-        <v>14850</v>
+        <v>18800</v>
       </c>
       <c r="D162" s="5">
         <f t="shared" si="16"/>
-        <v>2821.5</v>
+        <v>3572</v>
       </c>
       <c r="E162" s="9">
         <f t="shared" si="17"/>
-        <v>17671.5</v>
+        <v>22372</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A163" s="8" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C163" s="5">
-        <v>19800</v>
+        <v>21950</v>
       </c>
       <c r="D163" s="5">
         <f t="shared" si="16"/>
-        <v>3762</v>
+        <v>4170.5</v>
       </c>
       <c r="E163" s="9">
         <f t="shared" si="17"/>
-        <v>23562</v>
+        <v>26120.5</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A164" s="8" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B164" s="4" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="C164" s="5">
-        <v>15200</v>
+        <v>1600</v>
       </c>
       <c r="D164" s="5">
         <f t="shared" si="16"/>
-        <v>2888</v>
+        <v>304</v>
       </c>
       <c r="E164" s="9">
         <f t="shared" si="17"/>
-        <v>18088</v>
+        <v>1904</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A165" s="8" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B165" s="4" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C165" s="5">
-        <v>18800</v>
+        <v>3450</v>
       </c>
       <c r="D165" s="5">
         <f t="shared" si="16"/>
-        <v>3572</v>
+        <v>655.5</v>
       </c>
       <c r="E165" s="9">
         <f t="shared" si="17"/>
-        <v>22372</v>
+        <v>4105.5</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A166" s="8" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C166" s="5">
-        <v>21950</v>
+        <v>3850</v>
       </c>
       <c r="D166" s="5">
         <f t="shared" si="16"/>
-        <v>4170.5</v>
+        <v>731.5</v>
       </c>
       <c r="E166" s="9">
         <f t="shared" si="17"/>
-        <v>26120.5</v>
+        <v>4581.5</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A167" s="8" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B167" s="4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C167" s="5">
-        <v>1600</v>
+        <v>4800</v>
       </c>
       <c r="D167" s="5">
         <f t="shared" si="16"/>
-        <v>304</v>
+        <v>912</v>
       </c>
       <c r="E167" s="9">
         <f t="shared" si="17"/>
-        <v>1904</v>
+        <v>5712</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A168" s="8" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C168" s="5">
-        <v>3450</v>
+        <v>5450</v>
       </c>
       <c r="D168" s="5">
         <f t="shared" si="16"/>
-        <v>655.5</v>
+        <v>1035.5</v>
       </c>
       <c r="E168" s="9">
         <f t="shared" si="17"/>
-        <v>4105.5</v>
+        <v>6485.5</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A169" s="8" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B169" s="4" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C169" s="5">
-        <v>3850</v>
+        <v>5980</v>
       </c>
       <c r="D169" s="5">
         <f t="shared" si="16"/>
-        <v>731.5</v>
+        <v>1136.2</v>
       </c>
       <c r="E169" s="9">
         <f t="shared" si="17"/>
-        <v>4581.5</v>
+        <v>7116.2</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A170" s="8" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B170" s="4" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C170" s="5">
-        <v>4800</v>
+        <v>5730</v>
       </c>
       <c r="D170" s="5">
         <f t="shared" si="16"/>
-        <v>912</v>
+        <v>1088.7</v>
       </c>
       <c r="E170" s="9">
         <f t="shared" si="17"/>
-        <v>5712</v>
+        <v>6818.7</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A171" s="8" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B171" s="4" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C171" s="5">
-        <v>5450</v>
+        <v>6100</v>
       </c>
       <c r="D171" s="5">
         <f t="shared" si="16"/>
-        <v>1035.5</v>
+        <v>1159</v>
       </c>
       <c r="E171" s="9">
         <f t="shared" si="17"/>
-        <v>6485.5</v>
+        <v>7259</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A172" s="8" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B172" s="4" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C172" s="5">
-        <v>5980</v>
+        <v>9800</v>
       </c>
       <c r="D172" s="5">
         <f t="shared" si="16"/>
-        <v>1136.2</v>
+        <v>1862</v>
       </c>
       <c r="E172" s="9">
         <f t="shared" si="17"/>
-        <v>7116.2</v>
+        <v>11662</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A173" s="8" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B173" s="4" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="C173" s="5">
-        <v>5730</v>
+        <v>15850</v>
       </c>
       <c r="D173" s="5">
         <f t="shared" si="16"/>
-        <v>1088.7</v>
+        <v>3011.5</v>
       </c>
       <c r="E173" s="9">
         <f t="shared" si="17"/>
-        <v>6818.7</v>
+        <v>18861.5</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A174" s="8" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B174" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="C174" s="5">
-        <v>6100</v>
+        <v>14900</v>
       </c>
       <c r="D174" s="5">
         <f t="shared" si="16"/>
-        <v>1159</v>
+        <v>2831</v>
       </c>
       <c r="E174" s="9">
         <f t="shared" si="17"/>
-        <v>7259</v>
+        <v>17731</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A175" s="8" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="B175" s="4" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="C175" s="5">
-        <v>9800</v>
+        <v>21500</v>
       </c>
       <c r="D175" s="5">
         <f t="shared" si="16"/>
-        <v>1862</v>
+        <v>4085</v>
       </c>
       <c r="E175" s="9">
         <f t="shared" si="17"/>
-        <v>11662</v>
+        <v>25585</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A176" s="8" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B176" s="4" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C176" s="5">
-        <v>15850</v>
+        <v>27800</v>
       </c>
       <c r="D176" s="5">
         <f t="shared" si="16"/>
-        <v>3011.5</v>
+        <v>5282</v>
       </c>
       <c r="E176" s="9">
         <f t="shared" si="17"/>
-        <v>18861.5</v>
+        <v>33082</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A177" s="8" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B177" s="4" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C177" s="5">
-        <v>14900</v>
+        <v>19500</v>
       </c>
       <c r="D177" s="5">
         <f t="shared" si="16"/>
-        <v>2831</v>
+        <v>3705</v>
       </c>
       <c r="E177" s="9">
         <f t="shared" si="17"/>
-        <v>17731</v>
+        <v>23205</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A178" s="8" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C178" s="5">
-        <v>21500</v>
+        <v>10800</v>
       </c>
       <c r="D178" s="5">
         <f t="shared" si="16"/>
-        <v>4085</v>
+        <v>2052</v>
       </c>
       <c r="E178" s="9">
         <f t="shared" si="17"/>
-        <v>25585</v>
+        <v>12852</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A179" s="8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B179" s="4" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="C179" s="5">
-        <v>27800</v>
+        <v>7200</v>
       </c>
       <c r="D179" s="5">
         <f t="shared" si="16"/>
-        <v>5282</v>
+        <v>1368</v>
       </c>
       <c r="E179" s="9">
         <f t="shared" si="17"/>
-        <v>33082</v>
+        <v>8568</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A180" s="8" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B180" s="4" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C180" s="5">
-        <v>19500</v>
+        <v>5600</v>
       </c>
       <c r="D180" s="5">
         <f t="shared" si="16"/>
-        <v>3705</v>
+        <v>1064</v>
       </c>
       <c r="E180" s="9">
         <f t="shared" si="17"/>
-        <v>23205</v>
+        <v>6664</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A181" s="8" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C181" s="5">
-        <v>10800</v>
+        <v>10200</v>
       </c>
       <c r="D181" s="5">
         <f t="shared" si="16"/>
-        <v>2052</v>
+        <v>1938</v>
       </c>
       <c r="E181" s="9">
         <f t="shared" si="17"/>
-        <v>12852</v>
+        <v>12138</v>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A182" s="8" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B182" s="4" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="C182" s="5">
-        <v>7200</v>
+        <v>8250</v>
       </c>
       <c r="D182" s="5">
         <f t="shared" si="16"/>
-        <v>1368</v>
+        <v>1567.5</v>
       </c>
       <c r="E182" s="9">
         <f t="shared" si="17"/>
-        <v>8568</v>
+        <v>9817.5</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A183" s="8" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B183" s="4" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="C183" s="5">
-        <v>5600</v>
+        <v>6600</v>
       </c>
       <c r="D183" s="5">
         <f t="shared" si="16"/>
-        <v>1064</v>
+        <v>1254</v>
       </c>
       <c r="E183" s="9">
         <f t="shared" si="17"/>
-        <v>6664</v>
+        <v>7854</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A184" s="8" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C184" s="5">
-        <v>10200</v>
+        <v>10800</v>
       </c>
       <c r="D184" s="5">
         <f t="shared" si="16"/>
-        <v>1938</v>
+        <v>2052</v>
       </c>
       <c r="E184" s="9">
         <f t="shared" si="17"/>
-        <v>12138</v>
+        <v>12852</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A185" s="8" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B185" s="4" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C185" s="5">
-        <v>8250</v>
+        <v>8980</v>
       </c>
       <c r="D185" s="5">
         <f t="shared" si="16"/>
-        <v>1567.5</v>
+        <v>1706.2</v>
       </c>
       <c r="E185" s="9">
         <f t="shared" si="17"/>
-        <v>9817.5</v>
+        <v>10686.2</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A186" s="8" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="B186" s="4" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C186" s="5">
-        <v>6600</v>
+        <v>3100</v>
       </c>
       <c r="D186" s="5">
         <f t="shared" si="16"/>
-        <v>1254</v>
+        <v>589</v>
       </c>
       <c r="E186" s="9">
         <f t="shared" si="17"/>
-        <v>7854</v>
+        <v>3689</v>
       </c>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A187" s="8" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="B187" s="4" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C187" s="5">
-        <v>10800</v>
+        <v>10600</v>
       </c>
       <c r="D187" s="5">
         <f t="shared" si="16"/>
-        <v>2052</v>
+        <v>2014</v>
       </c>
       <c r="E187" s="9">
         <f t="shared" si="17"/>
-        <v>12852</v>
+        <v>12614</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A188" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B188" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C188" s="5">
-        <v>8980</v>
-      </c>
-      <c r="D188" s="5">
-        <f t="shared" si="16"/>
-        <v>1706.2</v>
-      </c>
-      <c r="E188" s="9">
-        <f t="shared" si="17"/>
-        <v>10686.2</v>
-      </c>
-    </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A189" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="B189" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C189" s="5">
-        <v>3100</v>
-      </c>
-      <c r="D189" s="5">
-        <f t="shared" si="16"/>
-        <v>589</v>
-      </c>
-      <c r="E189" s="9">
-        <f t="shared" si="17"/>
-        <v>3689</v>
-      </c>
+      <c r="A188" s="8"/>
+      <c r="B188" s="4"/>
+      <c r="C188" s="5"/>
+      <c r="D188" s="5"/>
+      <c r="E188" s="9"/>
+    </row>
+    <row r="189" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A189" s="23" t="s">
+        <v>261</v>
+      </c>
+      <c r="B189" s="24"/>
+      <c r="C189" s="24"/>
+      <c r="D189" s="24"/>
+      <c r="E189" s="25"/>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A190" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="B190" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C190" s="5">
-        <v>10600</v>
-      </c>
-      <c r="D190" s="5">
-        <f t="shared" si="16"/>
-        <v>2014</v>
-      </c>
-      <c r="E190" s="9">
-        <f t="shared" si="17"/>
-        <v>12614</v>
+      <c r="A190" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B190" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="C190" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D190" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E190" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A191" s="8"/>
-      <c r="B191" s="4"/>
-      <c r="C191" s="5"/>
-      <c r="D191" s="5"/>
-      <c r="E191" s="9"/>
-    </row>
-    <row r="192" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A192" s="23" t="s">
+      <c r="A191" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="B191" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="B192" s="24"/>
-      <c r="C192" s="24"/>
-      <c r="D192" s="24"/>
-      <c r="E192" s="25"/>
+      <c r="C191" s="5">
+        <v>4681</v>
+      </c>
+      <c r="D191" s="5">
+        <f t="shared" ref="D191:D198" si="18">C191*19%</f>
+        <v>889.39</v>
+      </c>
+      <c r="E191" s="9">
+        <f t="shared" ref="E191:E198" si="19">C191+D191</f>
+        <v>5570.39</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A192" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="B192" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="C192" s="5">
+        <v>7670</v>
+      </c>
+      <c r="D192" s="5">
+        <f t="shared" si="18"/>
+        <v>1457.3</v>
+      </c>
+      <c r="E192" s="9">
+        <f t="shared" si="19"/>
+        <v>9127.2999999999993</v>
+      </c>
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A193" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="B193" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="C193" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="D193" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E193" s="2" t="s">
-        <v>5</v>
+      <c r="A193" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="B193" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="C193" s="5">
+        <v>13130</v>
+      </c>
+      <c r="D193" s="5">
+        <f t="shared" si="18"/>
+        <v>2494.6999999999998</v>
+      </c>
+      <c r="E193" s="9">
+        <f t="shared" si="19"/>
+        <v>15624.7</v>
       </c>
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A194" s="8" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="B194" s="4" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="C194" s="5">
-        <v>4681</v>
+        <v>10400</v>
       </c>
       <c r="D194" s="5">
-        <f t="shared" ref="D194:D201" si="18">C194*19%</f>
-        <v>889.39</v>
+        <f t="shared" si="18"/>
+        <v>1976</v>
       </c>
       <c r="E194" s="9">
-        <f t="shared" ref="E194:E201" si="19">C194+D194</f>
-        <v>5570.39</v>
+        <f t="shared" si="19"/>
+        <v>12376</v>
       </c>
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A195" s="8" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B195" s="4" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C195" s="5">
-        <v>7670</v>
+        <v>8970</v>
       </c>
       <c r="D195" s="5">
         <f t="shared" si="18"/>
-        <v>1457.3</v>
+        <v>1704.3</v>
       </c>
       <c r="E195" s="9">
         <f t="shared" si="19"/>
-        <v>9127.2999999999993</v>
+        <v>10674.3</v>
       </c>
     </row>
     <row r="196" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A196" s="8" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="B196" s="4" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="C196" s="5">
-        <v>13130</v>
+        <v>7930</v>
       </c>
       <c r="D196" s="5">
         <f t="shared" si="18"/>
-        <v>2494.6999999999998</v>
+        <v>1506.7</v>
       </c>
       <c r="E196" s="9">
         <f t="shared" si="19"/>
-        <v>15624.7</v>
+        <v>9436.7000000000007</v>
       </c>
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A197" s="8" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="B197" s="4" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C197" s="5">
-        <v>10400</v>
+        <v>8060</v>
       </c>
       <c r="D197" s="5">
         <f t="shared" si="18"/>
-        <v>1976</v>
+        <v>1531.4</v>
       </c>
       <c r="E197" s="9">
         <f t="shared" si="19"/>
-        <v>12376</v>
+        <v>9591.4</v>
       </c>
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A198" s="8" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="B198" s="4" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="C198" s="5">
-        <v>8970</v>
+        <v>6110</v>
       </c>
       <c r="D198" s="5">
         <f t="shared" si="18"/>
-        <v>1704.3</v>
+        <v>1160.9000000000001</v>
       </c>
       <c r="E198" s="9">
         <f t="shared" si="19"/>
-        <v>10674.3</v>
-      </c>
-    </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A199" s="8" t="s">
-        <v>274</v>
-      </c>
-      <c r="B199" s="4" t="s">
-        <v>275</v>
-      </c>
-      <c r="C199" s="5">
-        <v>7930</v>
-      </c>
-      <c r="D199" s="5">
-        <f t="shared" si="18"/>
-        <v>1506.7</v>
-      </c>
-      <c r="E199" s="9">
-        <f t="shared" si="19"/>
-        <v>9436.7000000000007</v>
-      </c>
-    </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A200" s="8" t="s">
-        <v>276</v>
-      </c>
-      <c r="B200" s="4" t="s">
-        <v>277</v>
-      </c>
-      <c r="C200" s="5">
-        <v>8060</v>
-      </c>
-      <c r="D200" s="5">
-        <f t="shared" si="18"/>
-        <v>1531.4</v>
-      </c>
-      <c r="E200" s="9">
-        <f t="shared" si="19"/>
-        <v>9591.4</v>
-      </c>
-    </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A201" s="8" t="s">
-        <v>278</v>
-      </c>
-      <c r="B201" s="4" t="s">
-        <v>279</v>
-      </c>
-      <c r="C201" s="5">
-        <v>6110</v>
-      </c>
-      <c r="D201" s="5">
-        <f t="shared" si="18"/>
-        <v>1160.9000000000001</v>
-      </c>
-      <c r="E201" s="9">
-        <f t="shared" si="19"/>
         <v>7270.9</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A119:E119"/>
-    <mergeCell ref="A81:E81"/>
-    <mergeCell ref="A192:E192"/>
-    <mergeCell ref="A126:E126"/>
+    <mergeCell ref="A116:E116"/>
+    <mergeCell ref="A78:E78"/>
+    <mergeCell ref="A189:E189"/>
+    <mergeCell ref="A123:E123"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A152:E152"/>
+    <mergeCell ref="A149:E149"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4882,7 +4848,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>83</v>
@@ -4901,7 +4867,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>84</v>
@@ -6040,42 +6006,18 @@
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A78" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="B78" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="C78" s="5">
-        <v>2200</v>
-      </c>
-      <c r="D78" s="5">
-        <f>C78*19%</f>
-        <v>418</v>
-      </c>
-      <c r="E78" s="5">
-        <f>C78+D78</f>
-        <v>2618</v>
-      </c>
+      <c r="A78" s="3"/>
+      <c r="B78" s="4"/>
+      <c r="C78" s="5"/>
+      <c r="D78" s="5"/>
+      <c r="E78" s="5"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A79" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="B79" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="C79" s="5">
-        <v>2400</v>
-      </c>
-      <c r="D79" s="5">
-        <f>C79*19%</f>
-        <v>456</v>
-      </c>
-      <c r="E79" s="5">
-        <f>C79+D79</f>
-        <v>2856</v>
-      </c>
+      <c r="A79" s="3"/>
+      <c r="B79" s="4"/>
+      <c r="C79" s="5"/>
+      <c r="D79" s="5"/>
+      <c r="E79" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6099,7 +6041,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="26" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B1" s="27"/>
       <c r="C1" s="27"/>
@@ -6125,10 +6067,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C3" s="5">
         <v>2200</v>
@@ -6144,10 +6086,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C4" s="5">
         <v>2400</v>
@@ -6163,10 +6105,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C5" s="5">
         <v>1850</v>
@@ -6182,10 +6124,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C6" s="5">
         <v>4600</v>
@@ -6226,10 +6168,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C10" s="5">
         <v>2350</v>
@@ -6245,10 +6187,10 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="8" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C11" s="5">
         <v>2830</v>
@@ -6264,10 +6206,10 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="8" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C12" s="5">
         <v>3300</v>
@@ -6283,10 +6225,10 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="8" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C13" s="5">
         <v>3850</v>
@@ -6327,10 +6269,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="8" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C17" s="5">
         <v>7810</v>
@@ -6346,10 +6288,10 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="8" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C18" s="5">
         <v>8900</v>
@@ -6365,10 +6307,10 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="8" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C19" s="5">
         <v>10400</v>
@@ -6384,10 +6326,10 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="8" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C20" s="5">
         <v>12000</v>
@@ -6403,10 +6345,10 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="8" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C21" s="5">
         <v>19300</v>
@@ -6422,10 +6364,10 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="8" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C22" s="5">
         <v>22500</v>
@@ -6441,10 +6383,10 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="8" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C23" s="5">
         <v>26400</v>
@@ -6460,10 +6402,10 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="8" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C24" s="5">
         <v>28500</v>
@@ -6479,10 +6421,10 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="8" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C25" s="5">
         <v>31680</v>
@@ -6498,10 +6440,10 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="8" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C26" s="5">
         <v>40150</v>
@@ -6542,10 +6484,10 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="8" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C30" s="5">
         <v>17500</v>
@@ -6561,10 +6503,10 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="8" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C31" s="5">
         <v>25800</v>
@@ -6580,10 +6522,10 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="8" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C32" s="5">
         <v>29850</v>
@@ -6599,10 +6541,10 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" s="8" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C33" s="5">
         <v>32890</v>
@@ -6618,10 +6560,10 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="8" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C34" s="5">
         <v>38610</v>
@@ -6637,10 +6579,10 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="8" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C35" s="5">
         <v>48620</v>
@@ -6681,10 +6623,10 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" s="8" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C39" s="5">
         <v>55600</v>
@@ -6700,10 +6642,10 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" s="8" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C40" s="5">
         <v>60100</v>
@@ -6739,7 +6681,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="23" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B1" s="24"/>
       <c r="C1" s="24"/>
@@ -6765,10 +6707,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C3" s="5">
         <v>1500</v>
@@ -6784,10 +6726,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C4" s="5">
         <v>2600</v>
@@ -6803,10 +6745,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C5" s="5">
         <v>3700</v>
@@ -6822,10 +6764,10 @@
     </row>
     <row r="6" spans="1:5" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C6" s="13">
         <v>6500</v>
@@ -6861,7 +6803,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="20" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
@@ -6887,7 +6829,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>83</v>
@@ -6906,7 +6848,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>84</v>
@@ -8755,7 +8697,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="23" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B1" s="24"/>
       <c r="C1" s="24"/>
@@ -8781,10 +8723,10 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C3" s="5">
         <v>4681</v>
@@ -8800,10 +8742,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C4" s="5">
         <v>7670</v>
@@ -8819,10 +8761,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C5" s="5">
         <v>13130</v>
@@ -8838,10 +8780,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C6" s="5">
         <v>10400</v>
@@ -8857,10 +8799,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C7" s="5">
         <v>8970</v>
@@ -8876,10 +8818,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C8" s="5">
         <v>7930</v>
@@ -8895,10 +8837,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C9" s="5">
         <v>8060</v>
@@ -8914,10 +8856,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C10" s="5">
         <v>6110</v>

</xml_diff>

<commit_message>
Nosotros: imagen del banner CTA final cambiada a cta_footer_nosotros.jpg (optimizada 7MB→104KB)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_precios/Consolidado_lista_de_precios_2026_.xlsx
+++ b/_precios/Consolidado_lista_de_precios_2026_.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elcapel/Library/CloudStorage/GoogleDrive-garcia.persi@gmail.com/Mi unidad/KPL_BRANDING/Clientes/Devas/velas-devas/_precios/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elcapel/Library/CloudStorage/GoogleDrive-garcia.persi@gmail.com/Mi unidad/KPL_BRANDING/Clientes/Devas/Lista de precios Devas/2026_valores_reales/finales/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AECE92A-1A95-F149-8207-A935E826E258}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E8F9A94-5A09-7547-BF6D-16F2EE3C3E0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30240" yWindow="600" windowWidth="38400" windowHeight="21000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1440" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CONSOLIDADO" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="VELONES BANQUETERÍA" sheetId="5" r:id="rId5"/>
     <sheet name="PANTALLAS" sheetId="6" r:id="rId6"/>
     <sheet name="BANDEJAS" sheetId="7" r:id="rId7"/>
+    <sheet name="FUNERARIA" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="284">
   <si>
     <t>PANTALLAS</t>
   </si>
@@ -887,6 +888,9 @@
   </si>
   <si>
     <t>Velón 3,6x5</t>
+  </si>
+  <si>
+    <t>FUNERARIAS</t>
   </si>
 </sst>
 </file>
@@ -942,7 +946,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -962,7 +966,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -1231,11 +1235,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1290,11 +1309,44 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1305,12 +1357,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1636,13 +1682,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="22"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="32"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
@@ -1700,7 +1746,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="29" t="s">
         <v>279</v>
       </c>
       <c r="B6" s="4" t="s">
@@ -1776,7 +1822,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="30" t="s">
+      <c r="A10" s="29" t="s">
         <v>91</v>
       </c>
       <c r="B10" s="4" t="s">
@@ -1795,7 +1841,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="29" t="s">
         <v>93</v>
       </c>
       <c r="B11" s="4" t="s">
@@ -1814,7 +1860,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="29" t="s">
         <v>95</v>
       </c>
       <c r="B12" s="4" t="s">
@@ -1833,7 +1879,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="30" t="s">
+      <c r="A13" s="29" t="s">
         <v>97</v>
       </c>
       <c r="B13" s="4" t="s">
@@ -2289,7 +2335,7 @@
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" s="30" t="s">
+      <c r="A44" s="29" t="s">
         <v>145</v>
       </c>
       <c r="B44" s="4" t="s">
@@ -2308,7 +2354,7 @@
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" s="30" t="s">
+      <c r="A45" s="29" t="s">
         <v>147</v>
       </c>
       <c r="B45" s="4" t="s">
@@ -2841,13 +2887,13 @@
     </row>
     <row r="77" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="78" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="26" t="s">
+      <c r="A78" s="37" t="s">
         <v>205</v>
       </c>
-      <c r="B78" s="27"/>
-      <c r="C78" s="27"/>
-      <c r="D78" s="27"/>
-      <c r="E78" s="28"/>
+      <c r="B78" s="38"/>
+      <c r="C78" s="38"/>
+      <c r="D78" s="38"/>
+      <c r="E78" s="39"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" s="6" t="s">
@@ -3449,13 +3495,13 @@
       </c>
     </row>
     <row r="116" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A116" s="23" t="s">
+      <c r="A116" s="34" t="s">
         <v>254</v>
       </c>
-      <c r="B116" s="24"/>
-      <c r="C116" s="24"/>
-      <c r="D116" s="24"/>
-      <c r="E116" s="25"/>
+      <c r="B116" s="35"/>
+      <c r="C116" s="35"/>
+      <c r="D116" s="35"/>
+      <c r="E116" s="36"/>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A117" s="6" t="s">
@@ -3552,13 +3598,13 @@
     </row>
     <row r="122" spans="1:5" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="123" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A123" s="20" t="s">
+      <c r="A123" s="30" t="s">
         <v>260</v>
       </c>
-      <c r="B123" s="21"/>
-      <c r="C123" s="21"/>
-      <c r="D123" s="21"/>
-      <c r="E123" s="22"/>
+      <c r="B123" s="31"/>
+      <c r="C123" s="31"/>
+      <c r="D123" s="31"/>
+      <c r="E123" s="32"/>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" s="15" t="s">
@@ -3863,13 +3909,13 @@
       </c>
     </row>
     <row r="149" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A149" s="23" t="s">
+      <c r="A149" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B149" s="24"/>
-      <c r="C149" s="24"/>
-      <c r="D149" s="24"/>
-      <c r="E149" s="25"/>
+      <c r="B149" s="35"/>
+      <c r="C149" s="35"/>
+      <c r="D149" s="35"/>
+      <c r="E149" s="36"/>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A150" s="15" t="s">
@@ -4599,13 +4645,13 @@
       <c r="E188" s="9"/>
     </row>
     <row r="189" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A189" s="23" t="s">
+      <c r="A189" s="34" t="s">
         <v>261</v>
       </c>
-      <c r="B189" s="24"/>
-      <c r="C189" s="24"/>
-      <c r="D189" s="24"/>
-      <c r="E189" s="25"/>
+      <c r="B189" s="35"/>
+      <c r="C189" s="35"/>
+      <c r="D189" s="35"/>
+      <c r="E189" s="36"/>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A190" s="15" t="s">
@@ -4791,7 +4837,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E79"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.5" customWidth="1"/>
@@ -4802,13 +4848,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="22"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="32"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
@@ -4827,25 +4873,6 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="18" t="s">
-        <v>81</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="C3" s="17">
-        <v>480</v>
-      </c>
-      <c r="D3" s="5">
-        <f>C3*19%</f>
-        <v>91.2</v>
-      </c>
-      <c r="E3" s="5">
-        <f>C3+D3</f>
-        <v>571.20000000000005</v>
-      </c>
-    </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>278</v>
@@ -4857,11 +4884,11 @@
         <v>330</v>
       </c>
       <c r="D5" s="5">
-        <f t="shared" ref="D5:D14" si="0">C5*19%</f>
+        <f t="shared" ref="D5:D16" si="0">C5*19%</f>
         <v>62.7</v>
       </c>
       <c r="E5" s="5">
-        <f t="shared" ref="E5:E14" si="1">C5+D5</f>
+        <f t="shared" ref="E5:E16" si="1">C5+D5</f>
         <v>392.7</v>
       </c>
     </row>
@@ -4885,1139 +4912,1228 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B9" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C9" s="5">
         <v>580</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D9" s="5">
         <f t="shared" si="0"/>
         <v>110.2</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E9" s="5">
         <f t="shared" si="1"/>
         <v>690.2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B10" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C10" s="5">
         <v>890</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D10" s="5">
         <f t="shared" si="0"/>
         <v>169.1</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E10" s="5">
         <f t="shared" si="1"/>
         <v>1059.0999999999999</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B11" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C11" s="5">
         <v>1350</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D11" s="5">
         <f t="shared" si="0"/>
         <v>256.5</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E11" s="5">
         <f t="shared" si="1"/>
         <v>1606.5</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B12" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C12" s="5">
         <v>1420</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D12" s="5">
         <f t="shared" si="0"/>
         <v>269.8</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E12" s="5">
         <f t="shared" si="1"/>
         <v>1689.8</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B13" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C13" s="5">
         <v>2000</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D13" s="5">
         <f t="shared" si="0"/>
         <v>380</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E13" s="5">
         <f t="shared" si="1"/>
         <v>2380</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B14" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C14" s="5">
         <v>2400</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D14" s="5">
         <f t="shared" si="0"/>
         <v>456</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E14" s="5">
         <f t="shared" si="1"/>
         <v>2856</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B15" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C15" s="5">
         <v>2600</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D15" s="5">
         <f t="shared" si="0"/>
         <v>494</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E15" s="5">
         <f t="shared" si="1"/>
         <v>3094</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B16" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C16" s="5">
         <v>3580</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D16" s="5">
         <f t="shared" si="0"/>
         <v>680.2</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E16" s="5">
         <f t="shared" si="1"/>
         <v>4260.2</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="20"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B19" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C19" s="5">
         <v>1100</v>
       </c>
-      <c r="D16" s="5">
-        <f t="shared" ref="D16:D21" si="2">C16*19%</f>
+      <c r="D19" s="5">
+        <f t="shared" ref="D19:D24" si="2">C19*19%</f>
         <v>209</v>
       </c>
-      <c r="E16" s="5">
-        <f t="shared" ref="E16:E21" si="3">C16+D16</f>
+      <c r="E19" s="5">
+        <f t="shared" ref="E19:E24" si="3">C19+D19</f>
         <v>1309</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B20" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C20" s="5">
         <v>1700</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D20" s="5">
         <f t="shared" si="2"/>
         <v>323</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E20" s="5">
         <f t="shared" si="3"/>
         <v>2023</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B21" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="C18" s="5">
+      <c r="C21" s="5">
         <v>2250</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D21" s="5">
         <f t="shared" si="2"/>
         <v>427.5</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E21" s="5">
         <f t="shared" si="3"/>
         <v>2677.5</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B22" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="C19" s="5">
+      <c r="C22" s="5">
         <v>2680</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D22" s="5">
         <f t="shared" si="2"/>
         <v>509.2</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E22" s="5">
         <f t="shared" si="3"/>
         <v>3189.2</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B23" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="C20" s="5">
+      <c r="C23" s="5">
         <v>3390</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D23" s="5">
         <f t="shared" si="2"/>
         <v>644.1</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E23" s="5">
         <f t="shared" si="3"/>
         <v>4034.1</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="3" t="s">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B24" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="C21" s="5">
+      <c r="C24" s="5">
         <v>4500</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D24" s="5">
         <f t="shared" si="2"/>
         <v>855</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E24" s="5">
         <f t="shared" si="3"/>
         <v>5355</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C24" s="5">
-        <v>2530</v>
-      </c>
-      <c r="D24" s="5">
-        <f>C24*19%</f>
-        <v>480.7</v>
-      </c>
-      <c r="E24" s="5">
-        <f>C24+D24</f>
-        <v>3010.7</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C25" s="5">
-        <v>3100</v>
-      </c>
-      <c r="D25" s="5">
-        <f>C25*19%</f>
-        <v>589</v>
-      </c>
-      <c r="E25" s="5">
-        <f>C25+D25</f>
-        <v>3689</v>
-      </c>
-    </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C27" s="5">
-        <v>1380</v>
+        <v>2530</v>
       </c>
       <c r="D27" s="5">
         <f>C27*19%</f>
-        <v>262.2</v>
+        <v>480.7</v>
       </c>
       <c r="E27" s="5">
         <f>C27+D27</f>
+        <v>3010.7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C28" s="5">
+        <v>3100</v>
+      </c>
+      <c r="D28" s="5">
+        <f>C28*19%</f>
+        <v>589</v>
+      </c>
+      <c r="E28" s="5">
+        <f>C28+D28</f>
+        <v>3689</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="20"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C31" s="5">
+        <v>1380</v>
+      </c>
+      <c r="D31" s="5">
+        <f>C31*19%</f>
+        <v>262.2</v>
+      </c>
+      <c r="E31" s="5">
+        <f>C31+D31</f>
         <v>1642.2</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="3" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A32" s="20"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B34" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C29" s="5">
+      <c r="C34" s="5">
         <v>1680</v>
       </c>
-      <c r="D29" s="5">
-        <f t="shared" ref="D29:D34" si="4">C29*19%</f>
+      <c r="D34" s="5">
+        <f t="shared" ref="D34:D39" si="4">C34*19%</f>
         <v>319.2</v>
       </c>
-      <c r="E29" s="5">
-        <f t="shared" ref="E29:E34" si="5">C29+D29</f>
+      <c r="E34" s="5">
+        <f t="shared" ref="E34:E39" si="5">C34+D34</f>
         <v>1999.2</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="3" t="s">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B35" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="C30" s="5">
+      <c r="C35" s="5">
         <v>2700</v>
       </c>
-      <c r="D30" s="5">
+      <c r="D35" s="5">
         <f t="shared" si="4"/>
         <v>513</v>
       </c>
-      <c r="E30" s="5">
+      <c r="E35" s="5">
         <f t="shared" si="5"/>
         <v>3213</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="3" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B36" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="C31" s="5">
+      <c r="C36" s="5">
         <v>3340</v>
       </c>
-      <c r="D31" s="5">
+      <c r="D36" s="5">
         <f t="shared" si="4"/>
         <v>634.6</v>
       </c>
-      <c r="E31" s="5">
+      <c r="E36" s="5">
         <f t="shared" si="5"/>
         <v>3974.6</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="3" t="s">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B37" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="C32" s="5">
+      <c r="C37" s="5">
         <v>4180</v>
       </c>
-      <c r="D32" s="5">
+      <c r="D37" s="5">
         <f t="shared" si="4"/>
         <v>794.2</v>
       </c>
-      <c r="E32" s="5">
+      <c r="E37" s="5">
         <f t="shared" si="5"/>
         <v>4974.2</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="3" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B38" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="C33" s="5">
+      <c r="C38" s="5">
         <v>4950</v>
       </c>
-      <c r="D33" s="5">
+      <c r="D38" s="5">
         <f t="shared" si="4"/>
         <v>940.5</v>
       </c>
-      <c r="E33" s="5">
+      <c r="E38" s="5">
         <f t="shared" si="5"/>
         <v>5890.5</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" s="3" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B39" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="C34" s="5">
+      <c r="C39" s="5">
         <v>6680</v>
       </c>
-      <c r="D34" s="5">
+      <c r="D39" s="5">
         <f t="shared" si="4"/>
         <v>1269.2</v>
       </c>
-      <c r="E34" s="5">
+      <c r="E39" s="5">
         <f t="shared" si="5"/>
         <v>7949.2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="C36" s="5">
-        <v>2050</v>
-      </c>
-      <c r="D36" s="5">
-        <f>C36*19%</f>
-        <v>389.5</v>
-      </c>
-      <c r="E36" s="5">
-        <f>C36+D36</f>
-        <v>2439.5</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C37" s="5">
-        <v>3200</v>
-      </c>
-      <c r="D37" s="5">
-        <f>C37*19%</f>
-        <v>608</v>
-      </c>
-      <c r="E37" s="5">
-        <f>C37+D37</f>
-        <v>3808</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="C38" s="5">
-        <v>4100</v>
-      </c>
-      <c r="D38" s="5">
-        <f>C38*19%</f>
-        <v>779</v>
-      </c>
-      <c r="E38" s="5">
-        <f>C38+D38</f>
-        <v>4879</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="C39" s="5">
-        <v>5150</v>
-      </c>
-      <c r="D39" s="5">
-        <f>C39*19%</f>
-        <v>978.5</v>
-      </c>
-      <c r="E39" s="5">
-        <f>C39+D39</f>
-        <v>6128.5</v>
-      </c>
-    </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="C40" s="5">
-        <v>6100</v>
-      </c>
-      <c r="D40" s="5">
-        <f>C40*19%</f>
-        <v>1159</v>
-      </c>
-      <c r="E40" s="5">
-        <f>C40+D40</f>
-        <v>7259</v>
-      </c>
+      <c r="A40" s="20"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="22"/>
+      <c r="D40" s="22"/>
+      <c r="E40" s="22"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="C42" s="5">
-        <v>2200</v>
+        <v>2050</v>
       </c>
       <c r="D42" s="5">
-        <f t="shared" ref="D42:D53" si="6">C42*19%</f>
-        <v>418</v>
+        <f>C42*19%</f>
+        <v>389.5</v>
       </c>
       <c r="E42" s="5">
-        <f t="shared" ref="E42:E53" si="7">C42+D42</f>
-        <v>2618</v>
+        <f>C42+D42</f>
+        <v>2439.5</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C43" s="5">
+        <v>3200</v>
+      </c>
+      <c r="D43" s="5">
+        <f>C43*19%</f>
+        <v>608</v>
+      </c>
+      <c r="E43" s="5">
+        <f>C43+D43</f>
+        <v>3808</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C44" s="5">
+        <v>4100</v>
+      </c>
+      <c r="D44" s="5">
+        <f>C44*19%</f>
+        <v>779</v>
+      </c>
+      <c r="E44" s="5">
+        <f>C44+D44</f>
+        <v>4879</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C45" s="5">
+        <v>5150</v>
+      </c>
+      <c r="D45" s="5">
+        <f>C45*19%</f>
+        <v>978.5</v>
+      </c>
+      <c r="E45" s="5">
+        <f>C45+D45</f>
+        <v>6128.5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C46" s="5">
+        <v>6100</v>
+      </c>
+      <c r="D46" s="5">
+        <f>C46*19%</f>
+        <v>1159</v>
+      </c>
+      <c r="E46" s="5">
+        <f>C46+D46</f>
+        <v>7259</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" s="20"/>
+      <c r="B47" s="21"/>
+      <c r="C47" s="22"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="C49" s="5">
+        <v>2200</v>
+      </c>
+      <c r="D49" s="5">
+        <f t="shared" ref="D49:D60" si="6">C49*19%</f>
+        <v>418</v>
+      </c>
+      <c r="E49" s="5">
+        <f t="shared" ref="E49:E60" si="7">C49+D49</f>
+        <v>2618</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="B50" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="C43" s="5">
+      <c r="C50" s="5">
         <v>2750</v>
       </c>
-      <c r="D43" s="5">
+      <c r="D50" s="5">
         <f t="shared" si="6"/>
         <v>522.5</v>
       </c>
-      <c r="E43" s="5">
+      <c r="E50" s="5">
         <f t="shared" si="7"/>
         <v>3272.5</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" s="3" t="s">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="B44" s="4" t="s">
+      <c r="B51" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="C44" s="5">
+      <c r="C51" s="5">
         <v>4500</v>
       </c>
-      <c r="D44" s="5">
+      <c r="D51" s="5">
         <f t="shared" si="6"/>
         <v>855</v>
       </c>
-      <c r="E44" s="5">
+      <c r="E51" s="5">
         <f t="shared" si="7"/>
         <v>5355</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" s="3" t="s">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="B52" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="C45" s="5">
+      <c r="C52" s="5">
         <v>5450</v>
       </c>
-      <c r="D45" s="5">
+      <c r="D52" s="5">
         <f t="shared" si="6"/>
         <v>1035.5</v>
       </c>
-      <c r="E45" s="5">
+      <c r="E52" s="5">
         <f t="shared" si="7"/>
         <v>6485.5</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" s="3" t="s">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A53" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="B46" s="4" t="s">
+      <c r="B53" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="C46" s="5">
+      <c r="C53" s="5">
         <v>6850</v>
       </c>
-      <c r="D46" s="5">
+      <c r="D53" s="5">
         <f t="shared" si="6"/>
         <v>1301.5</v>
       </c>
-      <c r="E46" s="5">
+      <c r="E53" s="5">
         <f t="shared" si="7"/>
         <v>8151.5</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" s="3" t="s">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="B54" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="C47" s="5">
+      <c r="C54" s="5">
         <v>8100</v>
       </c>
-      <c r="D47" s="5">
+      <c r="D54" s="5">
         <f t="shared" si="6"/>
         <v>1539</v>
       </c>
-      <c r="E47" s="5">
+      <c r="E54" s="5">
         <f t="shared" si="7"/>
         <v>9639</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" s="3" t="s">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="B48" s="4" t="s">
+      <c r="B55" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="C48" s="5">
+      <c r="C55" s="5">
         <v>12100</v>
       </c>
-      <c r="D48" s="5">
+      <c r="D55" s="5">
         <f t="shared" si="6"/>
         <v>2299</v>
       </c>
-      <c r="E48" s="5">
+      <c r="E55" s="5">
         <f t="shared" si="7"/>
         <v>14399</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A49" s="3" t="s">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="B49" s="4" t="s">
+      <c r="B56" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="C49" s="5">
+      <c r="C56" s="5">
         <v>15200</v>
       </c>
-      <c r="D49" s="5">
+      <c r="D56" s="5">
         <f t="shared" si="6"/>
         <v>2888</v>
       </c>
-      <c r="E49" s="5">
+      <c r="E56" s="5">
         <f t="shared" si="7"/>
         <v>18088</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A50" s="3" t="s">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A57" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B57" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="C50" s="5">
+      <c r="C57" s="5">
         <v>18000</v>
       </c>
-      <c r="D50" s="5">
+      <c r="D57" s="5">
         <f t="shared" si="6"/>
         <v>3420</v>
       </c>
-      <c r="E50" s="5">
+      <c r="E57" s="5">
         <f t="shared" si="7"/>
         <v>21420</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A51" s="3" t="s">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A58" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B58" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="C51" s="5">
+      <c r="C58" s="5">
         <v>20900</v>
       </c>
-      <c r="D51" s="5">
+      <c r="D58" s="5">
         <f t="shared" si="6"/>
         <v>3971</v>
       </c>
-      <c r="E51" s="5">
+      <c r="E58" s="5">
         <f t="shared" si="7"/>
         <v>24871</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A52" s="3" t="s">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A59" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B59" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="C52" s="5">
+      <c r="C59" s="5">
         <v>24200</v>
       </c>
-      <c r="D52" s="5">
+      <c r="D59" s="5">
         <f t="shared" si="6"/>
         <v>4598</v>
       </c>
-      <c r="E52" s="5">
+      <c r="E59" s="5">
         <f t="shared" si="7"/>
         <v>28798</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A53" s="3" t="s">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A60" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="B53" s="4" t="s">
+      <c r="B60" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="C53" s="5">
+      <c r="C60" s="5">
         <v>30550</v>
       </c>
-      <c r="D53" s="5">
+      <c r="D60" s="5">
         <f t="shared" si="6"/>
         <v>5804.5</v>
       </c>
-      <c r="E53" s="5">
+      <c r="E60" s="5">
         <f t="shared" si="7"/>
         <v>36354.5</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A55" s="3" t="s">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A61" s="20"/>
+      <c r="B61" s="21"/>
+      <c r="C61" s="22"/>
+      <c r="D61" s="22"/>
+      <c r="E61" s="22"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A63" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B63" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="C55" s="5">
+      <c r="C63" s="5">
         <v>1550</v>
       </c>
-      <c r="D55" s="5">
-        <f>C55*19%</f>
+      <c r="D63" s="5">
+        <f>C63*19%</f>
         <v>294.5</v>
       </c>
-      <c r="E55" s="5">
-        <f>C55+D55</f>
+      <c r="E63" s="5">
+        <f>C63+D63</f>
         <v>1844.5</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A57" s="3" t="s">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A64" s="20"/>
+      <c r="B64" s="21"/>
+      <c r="C64" s="22"/>
+      <c r="D64" s="22"/>
+      <c r="E64" s="22"/>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A66" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="B57" s="4" t="s">
+      <c r="B66" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="C57" s="5">
+      <c r="C66" s="5">
         <v>3450</v>
       </c>
-      <c r="D57" s="5">
-        <f t="shared" ref="D57:D67" si="8">C57*19%</f>
+      <c r="D66" s="5">
+        <f t="shared" ref="D66:D76" si="8">C66*19%</f>
         <v>655.5</v>
       </c>
-      <c r="E57" s="5">
-        <f t="shared" ref="E57:E67" si="9">C57+D57</f>
+      <c r="E66" s="5">
+        <f t="shared" ref="E66:E76" si="9">C66+D66</f>
         <v>4105.5</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A58" s="3" t="s">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A67" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="B58" s="4" t="s">
+      <c r="B67" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="C58" s="5">
+      <c r="C67" s="5">
         <v>3650</v>
       </c>
-      <c r="D58" s="5">
+      <c r="D67" s="5">
         <f t="shared" si="8"/>
         <v>693.5</v>
       </c>
-      <c r="E58" s="5">
+      <c r="E67" s="5">
         <f t="shared" si="9"/>
         <v>4343.5</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A59" s="3" t="s">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A68" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="B68" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="C59" s="5">
+      <c r="C68" s="5">
         <v>5480</v>
       </c>
-      <c r="D59" s="5">
+      <c r="D68" s="5">
         <f t="shared" si="8"/>
         <v>1041.2</v>
       </c>
-      <c r="E59" s="5">
+      <c r="E68" s="5">
         <f t="shared" si="9"/>
         <v>6521.2</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A60" s="3" t="s">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A69" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="B60" s="4" t="s">
+      <c r="B69" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="C60" s="5">
+      <c r="C69" s="5">
         <v>7300</v>
       </c>
-      <c r="D60" s="5">
+      <c r="D69" s="5">
         <f t="shared" si="8"/>
         <v>1387</v>
       </c>
-      <c r="E60" s="5">
+      <c r="E69" s="5">
         <f t="shared" si="9"/>
         <v>8687</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A61" s="3" t="s">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A70" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="B61" s="4" t="s">
+      <c r="B70" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C61" s="5">
+      <c r="C70" s="5">
         <v>9130</v>
       </c>
-      <c r="D61" s="5">
+      <c r="D70" s="5">
         <f t="shared" si="8"/>
         <v>1734.7</v>
       </c>
-      <c r="E61" s="5">
+      <c r="E70" s="5">
         <f t="shared" si="9"/>
         <v>10864.7</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A62" s="3" t="s">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A71" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="B62" s="4" t="s">
+      <c r="B71" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C62" s="5">
+      <c r="C71" s="5">
         <v>10800</v>
       </c>
-      <c r="D62" s="5">
+      <c r="D71" s="5">
         <f t="shared" si="8"/>
         <v>2052</v>
       </c>
-      <c r="E62" s="5">
+      <c r="E71" s="5">
         <f t="shared" si="9"/>
         <v>12852</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A63" s="3" t="s">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A72" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="B63" s="4" t="s">
+      <c r="B72" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="C63" s="5">
+      <c r="C72" s="5">
         <v>16050</v>
       </c>
-      <c r="D63" s="5">
+      <c r="D72" s="5">
         <f t="shared" si="8"/>
         <v>3049.5</v>
       </c>
-      <c r="E63" s="5">
+      <c r="E72" s="5">
         <f t="shared" si="9"/>
         <v>19099.5</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A64" s="3" t="s">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A73" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="B64" s="4" t="s">
+      <c r="B73" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="C64" s="5">
+      <c r="C73" s="5">
         <v>20100</v>
       </c>
-      <c r="D64" s="5">
+      <c r="D73" s="5">
         <f t="shared" si="8"/>
         <v>3819</v>
       </c>
-      <c r="E64" s="5">
+      <c r="E73" s="5">
         <f t="shared" si="9"/>
         <v>23919</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A65" s="3" t="s">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A74" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="B65" s="4" t="s">
+      <c r="B74" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="C65" s="5">
+      <c r="C74" s="5">
         <v>23250</v>
       </c>
-      <c r="D65" s="5">
+      <c r="D74" s="5">
         <f t="shared" si="8"/>
         <v>4417.5</v>
       </c>
-      <c r="E65" s="5">
+      <c r="E74" s="5">
         <f t="shared" si="9"/>
         <v>27667.5</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A66" s="3" t="s">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A75" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="B66" s="4" t="s">
+      <c r="B75" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="C66" s="5">
+      <c r="C75" s="5">
         <v>32150</v>
       </c>
-      <c r="D66" s="5">
+      <c r="D75" s="5">
         <f t="shared" si="8"/>
         <v>6108.5</v>
       </c>
-      <c r="E66" s="5">
+      <c r="E75" s="5">
         <f t="shared" si="9"/>
         <v>38258.5</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A67" s="3" t="s">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A76" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="B67" s="4" t="s">
+      <c r="B76" s="4" t="s">
         <v>188</v>
       </c>
-      <c r="C67" s="5">
+      <c r="C76" s="5">
         <v>40000</v>
       </c>
-      <c r="D67" s="5">
+      <c r="D76" s="5">
         <f t="shared" si="8"/>
         <v>7600</v>
       </c>
-      <c r="E67" s="5">
+      <c r="E76" s="5">
         <f t="shared" si="9"/>
         <v>47600</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A69" s="3" t="s">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A77" s="20"/>
+      <c r="B77" s="21"/>
+      <c r="C77" s="22"/>
+      <c r="D77" s="22"/>
+      <c r="E77" s="22"/>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A79" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="B69" s="4" t="s">
+      <c r="B79" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="C69" s="5">
+      <c r="C79" s="5">
         <v>42000</v>
       </c>
-      <c r="D69" s="5">
-        <f>C69*19%</f>
+      <c r="D79" s="5">
+        <f>C79*19%</f>
         <v>7980</v>
       </c>
-      <c r="E69" s="5">
-        <f>C69+D69</f>
+      <c r="E79" s="5">
+        <f>C79+D79</f>
         <v>49980</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A70" s="3" t="s">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A80" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="B70" s="4" t="s">
+      <c r="B80" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="C70" s="5">
+      <c r="C80" s="5">
         <v>51500</v>
       </c>
-      <c r="D70" s="5">
-        <f>C70*19%</f>
+      <c r="D80" s="5">
+        <f>C80*19%</f>
         <v>9785</v>
       </c>
-      <c r="E70" s="5">
-        <f>C70+D70</f>
+      <c r="E80" s="5">
+        <f>C80+D80</f>
         <v>61285</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A72" s="3" t="s">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A81" s="20"/>
+      <c r="B81" s="21"/>
+      <c r="C81" s="22"/>
+      <c r="D81" s="22"/>
+      <c r="E81" s="22"/>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A83" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="B72" s="4" t="s">
+      <c r="B83" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="C72" s="5">
+      <c r="C83" s="5">
         <v>6450</v>
       </c>
-      <c r="D72" s="5">
-        <f>C72*19%</f>
+      <c r="D83" s="5">
+        <f>C83*19%</f>
         <v>1225.5</v>
       </c>
-      <c r="E72" s="5">
-        <f>C72+D72</f>
+      <c r="E83" s="5">
+        <f>C83+D83</f>
         <v>7675.5</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A73" s="3" t="s">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A84" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="B73" s="4" t="s">
+      <c r="B84" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="C73" s="5">
+      <c r="C84" s="5">
         <v>8800</v>
       </c>
-      <c r="D73" s="5">
-        <f>C73*19%</f>
+      <c r="D84" s="5">
+        <f>C84*19%</f>
         <v>1672</v>
       </c>
-      <c r="E73" s="5">
-        <f>C73+D73</f>
+      <c r="E84" s="5">
+        <f>C84+D84</f>
         <v>10472</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A74" s="3" t="s">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A85" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="B74" s="4" t="s">
+      <c r="B85" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="C74" s="5">
+      <c r="C85" s="5">
         <v>11500</v>
       </c>
-      <c r="D74" s="5">
-        <f>C74*19%</f>
+      <c r="D85" s="5">
+        <f>C85*19%</f>
         <v>2185</v>
       </c>
-      <c r="E74" s="5">
-        <f>C74+D74</f>
+      <c r="E85" s="5">
+        <f>C85+D85</f>
         <v>13685</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A75" s="3" t="s">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A86" s="23" t="s">
         <v>199</v>
       </c>
-      <c r="B75" s="4" t="s">
+      <c r="B86" s="24" t="s">
         <v>200</v>
       </c>
-      <c r="C75" s="5">
+      <c r="C86" s="25">
         <v>16000</v>
       </c>
-      <c r="D75" s="5">
-        <f>C75*19%</f>
+      <c r="D86" s="25">
+        <f>C86*19%</f>
         <v>3040</v>
       </c>
-      <c r="E75" s="5">
-        <f>C75+D75</f>
+      <c r="E86" s="25">
+        <f>C86+D86</f>
         <v>19040</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A76" s="3" t="s">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A87" s="26" t="s">
         <v>201</v>
       </c>
-      <c r="B76" s="4" t="s">
+      <c r="B87" s="27" t="s">
         <v>202</v>
       </c>
-      <c r="C76" s="5">
+      <c r="C87" s="28">
         <v>17600</v>
       </c>
-      <c r="D76" s="5">
-        <f>C76*19%</f>
+      <c r="D87" s="28">
+        <f>C87*19%</f>
         <v>3344</v>
       </c>
-      <c r="E76" s="5">
-        <f>C76+D76</f>
+      <c r="E87" s="28">
+        <f>C87+D87</f>
         <v>20944</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A78" s="3"/>
-      <c r="B78" s="4"/>
-      <c r="C78" s="5"/>
-      <c r="D78" s="5"/>
-      <c r="E78" s="5"/>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A79" s="3"/>
-      <c r="B79" s="4"/>
-      <c r="C79" s="5"/>
-      <c r="D79" s="5"/>
-      <c r="E79" s="5"/>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A89" s="20"/>
+      <c r="B89" s="21"/>
+      <c r="C89" s="22"/>
+      <c r="D89" s="22"/>
+      <c r="E89" s="22"/>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A90" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="B90" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C90" s="17">
+        <v>480</v>
+      </c>
+      <c r="D90" s="5">
+        <f>C90*19%</f>
+        <v>91.2</v>
+      </c>
+      <c r="E90" s="5">
+        <f>C90+D90</f>
+        <v>571.20000000000005</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6032,7 +6148,7 @@
   <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.1640625" customWidth="1"/>
+    <col min="1" max="1" width="24.5" customWidth="1"/>
     <col min="2" max="2" width="11.6640625" customWidth="1"/>
     <col min="3" max="3" width="15.83203125" customWidth="1"/>
     <col min="4" max="4" width="13.33203125" customWidth="1"/>
@@ -6040,13 +6156,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="37" t="s">
         <v>205</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="28"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="39"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -6105,7 +6221,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
-        <v>206</v>
+        <v>282</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>207</v>
@@ -6680,13 +6796,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="34" t="s">
         <v>254</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="25"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="36"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -6791,7 +6907,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.1640625" customWidth="1"/>
@@ -6802,13 +6918,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="30" t="s">
         <v>260</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="22"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="32"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
@@ -7079,7 +7195,7 @@
         <v>165</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C19" s="5">
         <v>1550</v>
@@ -7113,780 +7229,15 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B22" s="29"/>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
-      <c r="E22" s="29"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="23" t="s">
-        <v>0</v>
-      </c>
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="25"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="C24" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C25" s="5">
-        <v>1600</v>
-      </c>
-      <c r="D25" s="5">
-        <f t="shared" ref="D25:D37" si="2">C25*19%</f>
-        <v>304</v>
-      </c>
-      <c r="E25" s="9">
-        <f t="shared" ref="E25:E37" si="3">C25+D25</f>
-        <v>1904</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C26" s="5">
-        <v>2800</v>
-      </c>
-      <c r="D26" s="5">
-        <f t="shared" si="2"/>
-        <v>532</v>
-      </c>
-      <c r="E26" s="9">
-        <f t="shared" si="3"/>
-        <v>3332</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C27" s="5">
-        <v>3400</v>
-      </c>
-      <c r="D27" s="5">
-        <f t="shared" si="2"/>
-        <v>646</v>
-      </c>
-      <c r="E27" s="9">
-        <f t="shared" si="3"/>
-        <v>4046</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C28" s="5">
-        <v>4100</v>
-      </c>
-      <c r="D28" s="5">
-        <f t="shared" si="2"/>
-        <v>779</v>
-      </c>
-      <c r="E28" s="9">
-        <f t="shared" si="3"/>
-        <v>4879</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C29" s="5">
-        <v>5300</v>
-      </c>
-      <c r="D29" s="5">
-        <f t="shared" si="2"/>
-        <v>1007</v>
-      </c>
-      <c r="E29" s="9">
-        <f t="shared" si="3"/>
-        <v>6307</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C30" s="5">
-        <v>5800</v>
-      </c>
-      <c r="D30" s="5">
-        <f t="shared" si="2"/>
-        <v>1102</v>
-      </c>
-      <c r="E30" s="9">
-        <f t="shared" si="3"/>
-        <v>6902</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C31" s="5">
-        <v>5950</v>
-      </c>
-      <c r="D31" s="5">
-        <f t="shared" si="2"/>
-        <v>1130.5</v>
-      </c>
-      <c r="E31" s="9">
-        <f t="shared" si="3"/>
-        <v>7080.5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C32" s="5">
-        <v>9100</v>
-      </c>
-      <c r="D32" s="5">
-        <f t="shared" si="2"/>
-        <v>1729</v>
-      </c>
-      <c r="E32" s="9">
-        <f t="shared" si="3"/>
-        <v>10829</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C33" s="5">
-        <v>14850</v>
-      </c>
-      <c r="D33" s="5">
-        <f t="shared" si="2"/>
-        <v>2821.5</v>
-      </c>
-      <c r="E33" s="9">
-        <f t="shared" si="3"/>
-        <v>17671.5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C34" s="5">
-        <v>19800</v>
-      </c>
-      <c r="D34" s="5">
-        <f t="shared" si="2"/>
-        <v>3762</v>
-      </c>
-      <c r="E34" s="9">
-        <f t="shared" si="3"/>
-        <v>23562</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C35" s="5">
-        <v>15200</v>
-      </c>
-      <c r="D35" s="5">
-        <f t="shared" si="2"/>
-        <v>2888</v>
-      </c>
-      <c r="E35" s="9">
-        <f t="shared" si="3"/>
-        <v>18088</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C36" s="5">
-        <v>18800</v>
-      </c>
-      <c r="D36" s="5">
-        <f t="shared" si="2"/>
-        <v>3572</v>
-      </c>
-      <c r="E36" s="9">
-        <f t="shared" si="3"/>
-        <v>22372</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C37" s="5">
-        <v>21950</v>
-      </c>
-      <c r="D37" s="5">
-        <f t="shared" si="2"/>
-        <v>4170.5</v>
-      </c>
-      <c r="E37" s="9">
-        <f t="shared" si="3"/>
-        <v>26120.5</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" s="8"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="5"/>
-      <c r="E38" s="9"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C39" s="5">
-        <v>1600</v>
-      </c>
-      <c r="D39" s="5">
-        <f t="shared" ref="D39:D52" si="4">C39*19%</f>
-        <v>304</v>
-      </c>
-      <c r="E39" s="9">
-        <f t="shared" ref="E39:E52" si="5">C39+D39</f>
-        <v>1904</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C40" s="5">
-        <v>3450</v>
-      </c>
-      <c r="D40" s="5">
-        <f t="shared" si="4"/>
-        <v>655.5</v>
-      </c>
-      <c r="E40" s="9">
-        <f t="shared" si="5"/>
-        <v>4105.5</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C41" s="5">
-        <v>3850</v>
-      </c>
-      <c r="D41" s="5">
-        <f t="shared" si="4"/>
-        <v>731.5</v>
-      </c>
-      <c r="E41" s="9">
-        <f t="shared" si="5"/>
-        <v>4581.5</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C42" s="5">
-        <v>4800</v>
-      </c>
-      <c r="D42" s="5">
-        <f t="shared" si="4"/>
-        <v>912</v>
-      </c>
-      <c r="E42" s="9">
-        <f t="shared" si="5"/>
-        <v>5712</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C43" s="5">
-        <v>5450</v>
-      </c>
-      <c r="D43" s="5">
-        <f t="shared" si="4"/>
-        <v>1035.5</v>
-      </c>
-      <c r="E43" s="9">
-        <f t="shared" si="5"/>
-        <v>6485.5</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C44" s="5">
-        <v>5980</v>
-      </c>
-      <c r="D44" s="5">
-        <f t="shared" si="4"/>
-        <v>1136.2</v>
-      </c>
-      <c r="E44" s="9">
-        <f t="shared" si="5"/>
-        <v>7116.2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A45" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C45" s="5">
-        <v>5730</v>
-      </c>
-      <c r="D45" s="5">
-        <f t="shared" si="4"/>
-        <v>1088.7</v>
-      </c>
-      <c r="E45" s="9">
-        <f t="shared" si="5"/>
-        <v>6818.7</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C46" s="5">
-        <v>6100</v>
-      </c>
-      <c r="D46" s="5">
-        <f t="shared" si="4"/>
-        <v>1159</v>
-      </c>
-      <c r="E46" s="9">
-        <f t="shared" si="5"/>
-        <v>7259</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A47" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C47" s="5">
-        <v>9800</v>
-      </c>
-      <c r="D47" s="5">
-        <f t="shared" si="4"/>
-        <v>1862</v>
-      </c>
-      <c r="E47" s="9">
-        <f t="shared" si="5"/>
-        <v>11662</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C48" s="5">
-        <v>15850</v>
-      </c>
-      <c r="D48" s="5">
-        <f t="shared" si="4"/>
-        <v>3011.5</v>
-      </c>
-      <c r="E48" s="9">
-        <f t="shared" si="5"/>
-        <v>18861.5</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A49" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C49" s="5">
-        <v>14900</v>
-      </c>
-      <c r="D49" s="5">
-        <f t="shared" si="4"/>
-        <v>2831</v>
-      </c>
-      <c r="E49" s="9">
-        <f t="shared" si="5"/>
-        <v>17731</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A50" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C50" s="5">
-        <v>21500</v>
-      </c>
-      <c r="D50" s="5">
-        <f t="shared" si="4"/>
-        <v>4085</v>
-      </c>
-      <c r="E50" s="9">
-        <f t="shared" si="5"/>
-        <v>25585</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A51" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C51" s="5">
-        <v>27800</v>
-      </c>
-      <c r="D51" s="5">
-        <f t="shared" si="4"/>
-        <v>5282</v>
-      </c>
-      <c r="E51" s="9">
-        <f t="shared" si="5"/>
-        <v>33082</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A52" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C52" s="5">
-        <v>19500</v>
-      </c>
-      <c r="D52" s="5">
-        <f t="shared" si="4"/>
-        <v>3705</v>
-      </c>
-      <c r="E52" s="9">
-        <f t="shared" si="5"/>
-        <v>23205</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A53" s="8"/>
-      <c r="B53" s="4"/>
-      <c r="C53" s="5"/>
-      <c r="D53" s="5"/>
-      <c r="E53" s="9"/>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A54" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C54" s="5">
-        <v>10800</v>
-      </c>
-      <c r="D54" s="5">
-        <f>C54*19%</f>
-        <v>2052</v>
-      </c>
-      <c r="E54" s="9">
-        <f>C54+D54</f>
-        <v>12852</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A55" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C55" s="5">
-        <v>7200</v>
-      </c>
-      <c r="D55" s="5">
-        <f>C55*19%</f>
-        <v>1368</v>
-      </c>
-      <c r="E55" s="9">
-        <f>C55+D55</f>
-        <v>8568</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A56" s="8"/>
-      <c r="B56" s="4"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="5"/>
-      <c r="E56" s="9"/>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A57" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C57" s="5">
-        <v>5600</v>
-      </c>
-      <c r="D57" s="5">
-        <f>C57*19%</f>
-        <v>1064</v>
-      </c>
-      <c r="E57" s="9">
-        <f>C57+D57</f>
-        <v>6664</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A58" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="B58" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C58" s="5">
-        <v>10200</v>
-      </c>
-      <c r="D58" s="5">
-        <f>C58*19%</f>
-        <v>1938</v>
-      </c>
-      <c r="E58" s="9">
-        <f>C58+D58</f>
-        <v>12138</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A59" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C59" s="5">
-        <v>8250</v>
-      </c>
-      <c r="D59" s="5">
-        <f>C59*19%</f>
-        <v>1567.5</v>
-      </c>
-      <c r="E59" s="9">
-        <f>C59+D59</f>
-        <v>9817.5</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A60" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C60" s="5">
-        <v>6600</v>
-      </c>
-      <c r="D60" s="5">
-        <f>C60*19%</f>
-        <v>1254</v>
-      </c>
-      <c r="E60" s="9">
-        <f>C60+D60</f>
-        <v>7854</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A61" s="8"/>
-      <c r="B61" s="4"/>
-      <c r="C61" s="5"/>
-      <c r="D61" s="5"/>
-      <c r="E61" s="9"/>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A62" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="B62" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C62" s="5">
-        <v>10800</v>
-      </c>
-      <c r="D62" s="5">
-        <f>C62*19%</f>
-        <v>2052</v>
-      </c>
-      <c r="E62" s="9">
-        <f>C62+D62</f>
-        <v>12852</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A63" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B63" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C63" s="5">
-        <v>8980</v>
-      </c>
-      <c r="D63" s="5">
-        <f>C63*19%</f>
-        <v>1706.2</v>
-      </c>
-      <c r="E63" s="9">
-        <f>C63+D63</f>
-        <v>10686.2</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A64" s="8"/>
-      <c r="B64" s="4"/>
-      <c r="C64" s="5"/>
-      <c r="D64" s="5"/>
-      <c r="E64" s="9"/>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A65" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="B65" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C65" s="5">
-        <v>3100</v>
-      </c>
-      <c r="D65" s="5">
-        <f>C65*19%</f>
-        <v>589</v>
-      </c>
-      <c r="E65" s="9">
-        <f>C65+D65</f>
-        <v>3689</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A66" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="B66" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C66" s="5">
-        <v>10600</v>
-      </c>
-      <c r="D66" s="5">
-        <f>C66*19%</f>
-        <v>2014</v>
-      </c>
-      <c r="E66" s="9">
-        <f>C66+D66</f>
-        <v>12614</v>
-      </c>
+      <c r="B22" s="33"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="B22:E22"/>
-    <mergeCell ref="A23:E23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7905,13 +7256,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="25"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="36"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
@@ -8696,13 +8047,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="34" t="s">
         <v>261</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="25"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="36"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
@@ -8879,4 +8230,169 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABD0A7EF-727E-A942-8E81-5F403FE85B92}">
+  <dimension ref="A2:E11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="2" spans="1:5" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:5" ht="24" x14ac:dyDescent="0.2">
+      <c r="A3" s="30" t="s">
+        <v>283</v>
+      </c>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="32"/>
+    </row>
+    <row r="4" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A4" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="29" t="s">
+        <v>279</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="5">
+        <v>410</v>
+      </c>
+      <c r="D5" s="5">
+        <f t="shared" ref="D5" si="0">C5*19%</f>
+        <v>77.900000000000006</v>
+      </c>
+      <c r="E5" s="5">
+        <f t="shared" ref="E5" si="1">C5+D5</f>
+        <v>487.9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C6" s="5">
+        <v>1420</v>
+      </c>
+      <c r="D6" s="5">
+        <v>269.8</v>
+      </c>
+      <c r="E6" s="5">
+        <v>1689.8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="29" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" s="5">
+        <v>2000</v>
+      </c>
+      <c r="D7" s="5">
+        <v>380</v>
+      </c>
+      <c r="E7" s="5">
+        <v>2380</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="29" t="s">
+        <v>95</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C8" s="5">
+        <v>2400</v>
+      </c>
+      <c r="D8" s="5">
+        <v>456</v>
+      </c>
+      <c r="E8" s="5">
+        <v>2856</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="29" t="s">
+        <v>97</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C9" s="5">
+        <v>2600</v>
+      </c>
+      <c r="D9" s="5">
+        <v>494</v>
+      </c>
+      <c r="E9" s="5">
+        <v>3094</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="29" t="s">
+        <v>145</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C10" s="5">
+        <v>4500</v>
+      </c>
+      <c r="D10" s="5">
+        <f t="shared" ref="D10:D11" si="2">C10*19%</f>
+        <v>855</v>
+      </c>
+      <c r="E10" s="5">
+        <f t="shared" ref="E10:E11" si="3">C10+D10</f>
+        <v>5355</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="29" t="s">
+        <v>147</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C11" s="5">
+        <v>5450</v>
+      </c>
+      <c r="D11" s="5">
+        <f t="shared" si="2"/>
+        <v>1035.5</v>
+      </c>
+      <c r="E11" s="5">
+        <f t="shared" si="3"/>
+        <v>6485.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>